<commit_message>
Update Job Report Mon Jun  1 14:36:24 UTC 2026
</commit_message>
<xml_diff>
--- a/Latest_Job_Report.xlsx
+++ b/Latest_Job_Report.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI48"/>
+  <dimension ref="A1:AI51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -683,7 +683,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>li-4407427079</t>
+          <t>li-4404056876</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -693,27 +693,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407427079</t>
+          <t>https://www.linkedin.com/jobs/view/4404056876</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Research Scientist, Foundation Model</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Prior Labs</t>
+          <t>The IN Group</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46139</v>
+        <v>46170</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -732,7 +732,7 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/prior-labs</t>
+          <t>https://uk.linkedin.com/company/we-are-tig</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -1038,7 +1038,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>li-4404056876</t>
+          <t>li-4413434561</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1048,27 +1048,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404056876</t>
+          <t>https://www.linkedin.com/jobs/view/4413434561</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Research Assistant for Physics Laboratory (50%)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>The IN Group</t>
+          <t>University of Applied Sciences and Arts Northwestern Switzerland FHNW</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Windisch, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46170</v>
+        <v>46154</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1087,7 +1087,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/we-are-tig</t>
+          <t>https://ch.linkedin.com/school/fachhochschule-nordwestschweiz-fhnw/</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1109,7 +1109,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4413525792</t>
+          <t>li-4377188248</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1119,23 +1119,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413525792</t>
+          <t>https://www.linkedin.com/jobs/view/4377188248</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Market Researcher</t>
+          <t>Working Student - Executive Researcher 50% hybrid (m/f)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Xiaomi Technology</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Franke Group</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Aarburg, Aargau, Switzerland</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="n">
-        <v>46154</v>
+        <v>46162</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -1154,7 +1158,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
+          <t>https://ch.linkedin.com/company/franke-group</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1176,7 +1180,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4407397044</t>
+          <t>li-4404056876</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1186,27 +1190,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407397044</t>
+          <t>https://www.linkedin.com/jobs/view/4404056876</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Deutsches Diabetes-Zentrum</t>
+          <t>The IN Group</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46142</v>
+        <v>46170</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1225,7 +1229,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
+          <t>https://uk.linkedin.com/company/we-are-tig</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1247,7 +1251,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4257970631</t>
+          <t>li-4413525792</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1257,27 +1261,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4257970631</t>
+          <t>https://www.linkedin.com/jobs/view/4413525792</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
+          <t>Senior Market Researcher</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>WHU Entrepreneurship Roundtable</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Vallendar, Rhineland-Palatinate, Germany</t>
-        </is>
-      </c>
+          <t>Xiaomi Technology</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" s="2" t="n">
-        <v>45813</v>
+        <v>46154</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1296,7 +1296,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
+          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4412749267</t>
+          <t>li-4407397044</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1328,27 +1328,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412749267</t>
+          <t>https://www.linkedin.com/jobs/view/4407397044</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
+          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Carhartt WIP (Work In Progress)</t>
+          <t>Deutsches Diabetes-Zentrum</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46153</v>
+        <v>46142</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1367,7 +1367,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
+          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1383,13 +1383,13 @@
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr"/>
       <c r="AI12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>li-4417067089</t>
+          <t>li-4257970631</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1399,27 +1399,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4417067089</t>
+          <t>https://www.linkedin.com/jobs/view/4257970631</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Consultant / Manager Strategy Consulting</t>
+          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>LEAP PARTNERS</t>
+          <t>WHU Entrepreneurship Roundtable</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Vallendar, Rhineland-Palatinate, Germany</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46162</v>
+        <v>45813</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1438,7 +1438,7 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/leap-partners</t>
+          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -1454,13 +1454,13 @@
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>li-4409247899</t>
+          <t>li-4392923773</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1470,27 +1470,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409247899</t>
+          <t>https://www.linkedin.com/jobs/view/4392923773</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Content Specialist</t>
+          <t>Manager/in Operations (m/w/d)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>Thommen Group</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Aarwangen, Berne, Switzerland</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46149</v>
+        <v>46111</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1509,7 +1509,7 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://ch.linkedin.com/company/thommengroup</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -1602,7 +1602,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>li-4335125314</t>
+          <t>li-4409247899</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1612,27 +1612,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4335125314</t>
+          <t>https://www.linkedin.com/jobs/view/4409247899</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Consultant - Operations Excellence Program</t>
+          <t>Content Specialist</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46166</v>
+        <v>46149</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1651,7 +1651,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -1673,7 +1673,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>li-4335254607</t>
+          <t>li-4411718887</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1683,27 +1683,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4335254607</t>
+          <t>https://www.linkedin.com/jobs/view/4411718887</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Consultant - Procurement</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46166</v>
+        <v>46150</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1722,7 +1722,7 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -1744,7 +1744,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>li-4416102577</t>
+          <t>li-4412749267</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1754,27 +1754,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416102577</t>
+          <t>https://www.linkedin.com/jobs/view/4412749267</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Management Consultant</t>
+          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>Carhartt WIP (Work In Progress)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46162</v>
+        <v>46153</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1793,7 +1793,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -1886,7 +1886,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>li-4414574747</t>
+          <t>li-4417330465</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1896,27 +1896,27 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414574747</t>
+          <t>https://www.linkedin.com/jobs/view/4417330465</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Senior Cost Consultant</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Mace</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Belfort, Bourgogne-Franche-Comté, France</t>
+          <t>Breitenbach, Solothurn, Switzerland</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46156</v>
+        <v>46162</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1935,7 +1935,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://uk.linkedin.com/company/mace-group</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -1957,7 +1957,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>li-4416856371</t>
+          <t>li-4408692266</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1967,27 +1967,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416856371</t>
+          <t>https://www.linkedin.com/jobs/view/4408692266</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Filialleiter:in / Store Manager 100% - Basel</t>
+          <t>Country Sales Manager Schweiz (mwd)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Veloplus AG</t>
+          <t>CCR Commercial Refrigeration</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Pratteln, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46168</v>
+        <v>46146</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -2006,7 +2006,7 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/veloplus-ag</t>
+          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2028,7 +2028,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>li-4411456773</t>
+          <t>li-4416626453</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2038,27 +2038,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411456773</t>
+          <t>https://www.linkedin.com/jobs/view/4416626453</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>(Senior) Consultant Organisation &amp; Workforce Transformation</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46149</v>
+        <v>46161</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -2077,7 +2077,7 @@
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://www.linkedin.com/company/deloitte</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4416201877</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2109,27 +2109,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4416201877</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Supply Chain Planning Consultant</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46150</v>
+        <v>46160</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -2148,7 +2148,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://www.linkedin.com/company/deloitte</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2170,7 +2170,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>li-4398599784</t>
+          <t>li-4291106113</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2180,27 +2180,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4398599784</t>
+          <t>https://www.linkedin.com/jobs/view/4291106113</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Vice President, Business Manager</t>
+          <t>Consultant (m/f/d) - Financial Services</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AMETEK</t>
+          <t>Simon-Kucher</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Reinach, Basel-Country, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46162</v>
+        <v>46157</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -2219,7 +2219,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ametek</t>
+          <t>https://de.linkedin.com/company/simon-kucher</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2241,7 +2241,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>li-4408692266</t>
+          <t>li-4411456773</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4408692266</t>
+          <t>https://www.linkedin.com/jobs/view/4411456773</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Country Sales Manager Schweiz (mwd)</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>CCR Commercial Refrigeration</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Pratteln, Basel-Country, Switzerland</t>
+          <t>Colmar, Grand Est, France</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46146</v>
+        <v>46149</v>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -2290,7 +2290,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -2312,7 +2312,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>li-4392923773</t>
+          <t>li-4416856371</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2322,27 +2322,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4392923773</t>
+          <t>https://www.linkedin.com/jobs/view/4416856371</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Manager/in Operations (m/w/d)</t>
+          <t>Filialleiter:in / Store Manager 100% - Basel</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Thommen Group</t>
+          <t>Veloplus AG</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Aarwangen, Berne, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46111</v>
+        <v>46168</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -2361,7 +2361,7 @@
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/thommengroup</t>
+          <t>https://ch.linkedin.com/company/veloplus-ag</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -2450,7 +2450,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>li-4416485748</t>
+          <t>li-4398599784</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2460,27 +2460,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416485748</t>
+          <t>https://www.linkedin.com/jobs/view/4398599784</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Drug Safety Case Manager</t>
+          <t>Vice President, Business Manager</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Flexsis</t>
+          <t>AMETEK</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Allschwil, Basel-Country, Switzerland</t>
+          <t>Reinach, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -2499,7 +2499,7 @@
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/flexsisch</t>
+          <t>https://www.linkedin.com/company/ametek</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -2521,7 +2521,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4421813206</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2531,28 +2531,26 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4421813206</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Business / Senior Consultant</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>MAK Consulting AG</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>46150</v>
-      </c>
+          <t>Zollikofen, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -2570,7 +2568,7 @@
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://ch.linkedin.com/company/mak-consulting-ag</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -2663,7 +2661,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>li-4301569738</t>
+          <t>li-4411984255</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2673,27 +2671,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4301569738</t>
+          <t>https://www.linkedin.com/jobs/view/4411984255</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Experienced Consultant - Capital Excellence</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46173</v>
+        <v>46151</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -2712,7 +2710,7 @@
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W31" t="inlineStr"/>
@@ -2734,7 +2732,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>li-4415258961</t>
+          <t>li-4410039212</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2744,27 +2742,23 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4415258961</t>
+          <t>https://www.linkedin.com/jobs/view/4410039212</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Strategy Consultant</t>
+          <t>Country Manager Germany</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Anding &amp; Company</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
+          <t>DeWarmte</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" s="2" t="n">
-        <v>46168</v>
+        <v>46146</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -2783,7 +2777,7 @@
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/andingandcompany</t>
+          <t>https://nl.linkedin.com/company/dewarmte</t>
         </is>
       </c>
       <c r="W32" t="inlineStr"/>
@@ -2805,7 +2799,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>li-4266954854</t>
+          <t>li-4412263197</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2815,23 +2809,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4266954854</t>
+          <t>https://www.linkedin.com/jobs/view/4412263197</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Experienced Consultant (Düsseldorf)</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>OC&amp;C Strategy Consultants</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>SThree</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
       <c r="H33" s="2" t="n">
-        <v>46161</v>
+        <v>46160</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -2850,7 +2848,7 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/oc&amp;c-strategy-consultants</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W33" t="inlineStr"/>
@@ -2872,7 +2870,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>li-4301586122</t>
+          <t>li-4412289349</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2882,18 +2880,18 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4301586122</t>
+          <t>https://www.linkedin.com/jobs/view/4412289349</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Experienced Consultant - Capital Excellence</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>SThree</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2902,7 +2900,7 @@
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46154</v>
+        <v>46160</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -2921,7 +2919,7 @@
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W34" t="inlineStr"/>
@@ -2943,7 +2941,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>li-4371968232</t>
+          <t>li-4410012963</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2953,18 +2951,18 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4371968232</t>
+          <t>https://www.linkedin.com/jobs/view/4410012963</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Consultant (w/m/d) Public Sector</t>
+          <t>Senior Associate - Consulting</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Horváth</t>
+          <t>VIVALDI_</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2973,7 +2971,7 @@
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>46070</v>
+        <v>46121</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
@@ -2992,7 +2990,7 @@
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/horvathpartners</t>
+          <t>https://www.linkedin.com/company/vivaldi-group</t>
         </is>
       </c>
       <c r="W35" t="inlineStr"/>
@@ -3014,7 +3012,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>li-4416894948</t>
+          <t>li-4389002832</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3024,27 +3022,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416894948</t>
+          <t>https://www.linkedin.com/jobs/view/4389002832</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Spezialist (m/w/d) für Einlagensicherung</t>
+          <t>Management Consultant (d/f/m), DHL Consulting Europe</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Prüfungsverband deutscher Banken e.V.</t>
+          <t>DHL</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>46169</v>
+        <v>46105</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -3063,7 +3061,7 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/pruefungsverbanddeutscherbanken</t>
+          <t>https://de.linkedin.com/company/dhl</t>
         </is>
       </c>
       <c r="W36" t="inlineStr"/>
@@ -3085,7 +3083,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>li-4421807992</t>
+          <t>li-4048085587</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3095,26 +3093,28 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4421807992</t>
+          <t>https://www.linkedin.com/jobs/view/4048085587</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Revisor Specialist - Penny International (m/w/d)</t>
+          <t>(Junior) Consultant (w/m/d) Banking &amp; Financial Institutions</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>PENNY International (REWE Group)</t>
+          <t>Horváth</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>45580</v>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
@@ -3132,7 +3132,7 @@
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/penny-international-rewe-group</t>
+          <t>https://de.linkedin.com/company/horvathpartners</t>
         </is>
       </c>
       <c r="W37" t="inlineStr"/>
@@ -3154,7 +3154,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>li-4404077580</t>
+          <t>li-4384316600</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3164,27 +3164,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404077580</t>
+          <t>https://www.linkedin.com/jobs/view/4384316600</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - Post Training</t>
+          <t>Sales Area Manager Nürnberg Würzburg (w_m_d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Black Forest Labs</t>
+          <t>Barilla Group</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>46132</v>
+        <v>46157</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -3203,7 +3203,7 @@
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/bflai</t>
+          <t>https://it.linkedin.com/company/barilla-group</t>
         </is>
       </c>
       <c r="W38" t="inlineStr"/>
@@ -3225,7 +3225,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>li-4404067638</t>
+          <t>li-4413931472</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3235,27 +3235,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404067638</t>
+          <t>https://www.linkedin.com/jobs/view/4413931472</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - VLM</t>
+          <t>Store Manager (m/w/d), Emporio Armani Düsseldorf</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Black Forest Labs</t>
+          <t>Giorgio Armani</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46132</v>
+        <v>46155</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -3274,7 +3274,7 @@
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/bflai</t>
+          <t>https://it.linkedin.com/company/giorgio-armani</t>
         </is>
       </c>
       <c r="W39" t="inlineStr"/>
@@ -3296,7 +3296,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>li-4404071603</t>
+          <t>li-4411814591</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3306,27 +3306,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404071603</t>
+          <t>https://www.linkedin.com/jobs/view/4411814591</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - Pretraining</t>
+          <t>General Manager (STARS)*</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Black Forest Labs</t>
+          <t>tristar Hotels</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Monheim, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>46132</v>
+        <v>46149</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -3345,7 +3345,7 @@
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/bflai</t>
+          <t>https://de.linkedin.com/company/tristarhotels</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
@@ -3367,7 +3367,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>li-4315852967</t>
+          <t>li-4379922140</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3377,27 +3377,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4315852967</t>
+          <t>https://www.linkedin.com/jobs/view/4379922140</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - Image / Video Generation</t>
+          <t>Area Manager - Cologne (m/f/d)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Black Forest Labs</t>
+          <t>LAP Coffee</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>45946</v>
+        <v>46083</v>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
@@ -3416,7 +3416,7 @@
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/bflai</t>
+          <t>https://de.linkedin.com/company/lap-coffee</t>
         </is>
       </c>
       <c r="W41" t="inlineStr"/>
@@ -3438,7 +3438,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>li-4414586149</t>
+          <t>li-4411990173</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414586149</t>
+          <t>https://www.linkedin.com/jobs/view/4411990173</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -3464,11 +3464,11 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>46156</v>
+        <v>46151</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -3509,7 +3509,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>li-4411991147</t>
+          <t>li-4407754531</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3519,27 +3519,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411991147</t>
+          <t>https://www.linkedin.com/jobs/view/4407754531</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Supply Chain Lead (gn) bei SAMSUNG</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Grafton Recruitment</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>46151</v>
+        <v>46164</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -3558,7 +3558,7 @@
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://it.linkedin.com/company/grafton-recruitment</t>
         </is>
       </c>
       <c r="W43" t="inlineStr"/>
@@ -3580,7 +3580,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>li-4411990173</t>
+          <t>li-4412263197</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3590,27 +3590,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411990173</t>
+          <t>https://www.linkedin.com/jobs/view/4412263197</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>SThree</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>46151</v>
+        <v>46160</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -3629,7 +3629,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W44" t="inlineStr"/>
@@ -3651,7 +3651,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>li-4411984255</t>
+          <t>li-4412289349</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3661,27 +3661,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411984255</t>
+          <t>https://www.linkedin.com/jobs/view/4412289349</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>SThree</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>46151</v>
+        <v>46160</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -3700,7 +3700,7 @@
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W45" t="inlineStr"/>
@@ -3722,7 +3722,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>li-4411456773</t>
+          <t>li-4416248930</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3732,27 +3732,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411456773</t>
+          <t>https://www.linkedin.com/jobs/view/4416248930</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Ostendorf Consulting</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H46" s="2" t="n">
-        <v>46149</v>
+        <v>46160</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://de.linkedin.com/company/ostendorf-consulting</t>
         </is>
       </c>
       <c r="W46" t="inlineStr"/>
@@ -3793,7 +3793,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>li-4417604986</t>
+          <t>li-4409342469</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3803,27 +3803,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4417604986</t>
+          <t>https://www.linkedin.com/jobs/view/4409342469</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Facility Coordinator (a) 80%</t>
+          <t>Customer Onboarding Specialist</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>JYSK</t>
+          <t>eviivo</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Zofingen, Aargau, Switzerland</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H47" s="2" t="n">
-        <v>46170</v>
+        <v>46147</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
@@ -3842,7 +3842,7 @@
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/company/jysk</t>
+          <t>https://uk.linkedin.com/company/eviivo</t>
         </is>
       </c>
       <c r="W47" t="inlineStr"/>
@@ -3864,7 +3864,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>li-4386750509</t>
+          <t>li-4411718887</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3874,27 +3874,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386750509</t>
+          <t>https://www.linkedin.com/jobs/view/4411718887</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Spontanbewerbung</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>INFORS HT</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Bottmingen, Basel-Country, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H48" s="2" t="n">
-        <v>46098</v>
+        <v>46150</v>
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
@@ -3913,7 +3913,7 @@
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/inforsht</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W48" t="inlineStr"/>
@@ -3932,6 +3932,219 @@
         <v>0</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>li-4404786229</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4404786229</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Fraunhofer IAF</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="b">
+        <v>0</v>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr"/>
+      <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr"/>
+      <c r="AI49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>li-4411991147</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4411991147</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Strasbourg, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>46151</v>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="b">
+        <v>0</v>
+      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr"/>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>li-4386750509</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4386750509</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Spontanbewerbung</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>INFORS HT</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Bottmingen, Basel-Country, Switzerland</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="b">
+        <v>0</v>
+      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>https://ch.linkedin.com/company/inforsht</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="inlineStr"/>
+      <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr"/>
+      <c r="AI51" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Job Report Mon Jun  1 14:51:14 UTC 2026
</commit_message>
<xml_diff>
--- a/Latest_Job_Report.xlsx
+++ b/Latest_Job_Report.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI51"/>
+  <dimension ref="A1:AI46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -754,7 +754,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>li-4415995749</t>
+          <t>li-4413525792</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -764,27 +764,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4415995749</t>
+          <t>https://www.linkedin.com/jobs/view/4413525792</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Investment Research Analyst</t>
+          <t>Senior Market Researcher</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Mercor</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Zurich, Zurich, Switzerland</t>
-        </is>
-      </c>
+          <t>Xiaomi Technology</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" s="2" t="n">
-        <v>46162</v>
+        <v>46154</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -803,7 +799,7 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -825,7 +821,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>li-4418110532</t>
+          <t>li-4407397044</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -835,27 +831,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4418110532</t>
+          <t>https://www.linkedin.com/jobs/view/4407397044</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Medical Researcher (m/w/d)</t>
+          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Deutsches Promotionszentrum</t>
+          <t>Deutsches Diabetes-Zentrum</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46164</v>
+        <v>46142</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -874,7 +870,7 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
+          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -896,7 +892,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>li-4414173590</t>
+          <t>li-4257970631</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -906,27 +902,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414173590</t>
+          <t>https://www.linkedin.com/jobs/view/4257970631</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Investment Research Analyst | Upto $100/hr</t>
+          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>WHU Entrepreneurship Roundtable</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Vallendar, Rhineland-Palatinate, Germany</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46155</v>
+        <v>45813</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -945,7 +941,7 @@
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -967,7 +963,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>li-4410472579</t>
+          <t>li-4418110532</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -977,27 +973,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410472579</t>
+          <t>https://www.linkedin.com/jobs/view/4418110532</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Quantitative Researcher</t>
+          <t>Medical Researcher (m/w/d)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>STS Digital Group</t>
+          <t>Deutsches Promotionszentrum</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46149</v>
+        <v>46164</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -1016,7 +1012,7 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sts-digital-group</t>
+          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1038,7 +1034,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>li-4413434561</t>
+          <t>li-4404056876</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1048,27 +1044,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413434561</t>
+          <t>https://www.linkedin.com/jobs/view/4404056876</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Research Assistant for Physics Laboratory (50%)</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>University of Applied Sciences and Arts Northwestern Switzerland FHNW</t>
+          <t>The IN Group</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Windisch, Aargau, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46154</v>
+        <v>46170</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1087,7 +1083,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/school/fachhochschule-nordwestschweiz-fhnw/</t>
+          <t>https://uk.linkedin.com/company/we-are-tig</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1109,7 +1105,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4377188248</t>
+          <t>li-4415995749</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1119,23 +1115,23 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4377188248</t>
+          <t>https://www.linkedin.com/jobs/view/4415995749</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Working Student - Executive Researcher 50% hybrid (m/f)</t>
+          <t>Investment Research Analyst</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Franke Group</t>
+          <t>Mercor</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Aarburg, Aargau, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1158,7 +1154,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/franke-group</t>
+          <t>https://www.linkedin.com/company/mercor-ai</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1180,7 +1176,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4404056876</t>
+          <t>li-4414173590</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1190,27 +1186,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404056876</t>
+          <t>https://www.linkedin.com/jobs/view/4414173590</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Investment Research Analyst | Upto $100/hr</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>The IN Group</t>
+          <t>Mercor</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46170</v>
+        <v>46155</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1229,7 +1225,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/we-are-tig</t>
+          <t>https://www.linkedin.com/company/mercor-ai</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1251,7 +1247,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4413525792</t>
+          <t>li-4410472579</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1261,23 +1257,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413525792</t>
+          <t>https://www.linkedin.com/jobs/view/4410472579</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Market Researcher</t>
+          <t>Quantitative Researcher</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Xiaomi Technology</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>STS Digital Group</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="n">
-        <v>46154</v>
+        <v>46149</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1296,7 +1296,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
+          <t>https://www.linkedin.com/company/sts-digital-group</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4407397044</t>
+          <t>li-4413434561</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1328,27 +1328,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407397044</t>
+          <t>https://www.linkedin.com/jobs/view/4413434561</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
+          <t>Research Assistant for Physics Laboratory (50%)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Deutsches Diabetes-Zentrum</t>
+          <t>University of Applied Sciences and Arts Northwestern Switzerland FHNW</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Windisch, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46142</v>
+        <v>46154</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1367,7 +1367,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
+          <t>https://ch.linkedin.com/school/fachhochschule-nordwestschweiz-fhnw/</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1389,7 +1389,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>li-4257970631</t>
+          <t>li-4377188248</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1399,27 +1399,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4257970631</t>
+          <t>https://www.linkedin.com/jobs/view/4377188248</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
+          <t>Working Student - Executive Researcher 50% hybrid (m/f)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>WHU Entrepreneurship Roundtable</t>
+          <t>Franke Group</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Vallendar, Rhineland-Palatinate, Germany</t>
+          <t>Aarburg, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>45813</v>
+        <v>46162</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1438,7 +1438,7 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
+          <t>https://ch.linkedin.com/company/franke-group</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -1460,7 +1460,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>li-4392923773</t>
+          <t>li-4409306761</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1470,27 +1470,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4392923773</t>
+          <t>https://www.linkedin.com/jobs/view/4409306761</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Manager/in Operations (m/w/d)</t>
+          <t>Country Manager Belgium and Luxembourg (BeLux-based) 🇧🇪🇱🇺</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Thommen Group</t>
+          <t>Chargemap</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Aarwangen, Berne, Switzerland</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46111</v>
+        <v>46147</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1509,7 +1509,7 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/thommengroup</t>
+          <t>https://fr.linkedin.com/company/chargemap</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -1531,7 +1531,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>li-4404786229</t>
+          <t>li-4408692266</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1541,27 +1541,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404786229</t>
+          <t>https://www.linkedin.com/jobs/view/4408692266</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
+          <t>Country Sales Manager Schweiz (mwd)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Fraunhofer IAF</t>
+          <t>CCR Commercial Refrigeration</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Pratteln, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46135</v>
+        <v>46146</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1580,7 +1580,7 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
+          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -1602,7 +1602,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>li-4409247899</t>
+          <t>li-4335125314</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1612,27 +1612,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409247899</t>
+          <t>https://www.linkedin.com/jobs/view/4335125314</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Content Specialist</t>
+          <t>Consultant - Operations Excellence Program</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46149</v>
+        <v>46166</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1651,7 +1651,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -1673,7 +1673,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4404786229</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1683,27 +1683,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4404786229</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>Fraunhofer IAF</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46150</v>
+        <v>46135</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1722,7 +1722,7 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -1744,7 +1744,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>li-4412749267</t>
+          <t>li-4413366651</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1754,27 +1754,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412749267</t>
+          <t>https://www.linkedin.com/jobs/view/4413366651</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
+          <t>Assistant General Manager / Assistenz der Hoteldirektion (m/w/d)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Carhartt WIP (Work In Progress)</t>
+          <t>Hotel Am Rathaus Freibug</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46153</v>
+        <v>46162</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1793,7 +1793,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
+          <t>https://www.linkedin.com/company/hotel-am-rathaus-freibug</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -1815,7 +1815,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>li-4416485748</t>
+          <t>li-4335254607</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1825,27 +1825,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416485748</t>
+          <t>https://www.linkedin.com/jobs/view/4335254607</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Drug Safety Case Manager</t>
+          <t>Consultant - Procurement</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Flexsis</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Allschwil, Basel-Country, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46161</v>
+        <v>46166</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1864,7 +1864,7 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/flexsisch</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -1886,7 +1886,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>li-4417330465</t>
+          <t>li-4417067089</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1896,23 +1896,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4417330465</t>
+          <t>https://www.linkedin.com/jobs/view/4417067089</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Cost Consultant</t>
+          <t>Senior Consultant / Manager Strategy Consulting</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Mace</t>
+          <t>LEAP PARTNERS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Breitenbach, Solothurn, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1935,7 +1935,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/mace-group</t>
+          <t>https://ch.linkedin.com/company/leap-partners</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -1957,7 +1957,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>li-4408692266</t>
+          <t>li-4416102577</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1967,27 +1967,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4408692266</t>
+          <t>https://www.linkedin.com/jobs/view/4416102577</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Country Sales Manager Schweiz (mwd)</t>
+          <t>Management Consultant</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CCR Commercial Refrigeration</t>
+          <t>Mercor</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Pratteln, Basel-Country, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46146</v>
+        <v>46162</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -2006,7 +2006,7 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
+          <t>https://www.linkedin.com/company/mercor-ai</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2028,7 +2028,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>li-4416626453</t>
+          <t>li-4414574747</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2038,27 +2038,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416626453</t>
+          <t>https://www.linkedin.com/jobs/view/4414574747</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>(Senior) Consultant Organisation &amp; Workforce Transformation</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Belfort, Bourgogne-Franche-Comté, France</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46161</v>
+        <v>46156</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -2077,7 +2077,7 @@
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deloitte</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>li-4416201877</t>
+          <t>li-4416485748</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2109,27 +2109,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416201877</t>
+          <t>https://www.linkedin.com/jobs/view/4416485748</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Supply Chain Planning Consultant</t>
+          <t>Drug Safety Case Manager</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Flexsis</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Allschwil, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -2148,7 +2148,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deloitte</t>
+          <t>https://ch.linkedin.com/company/flexsisch</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2170,7 +2170,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>li-4291106113</t>
+          <t>li-4412749267</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2180,27 +2180,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4291106113</t>
+          <t>https://www.linkedin.com/jobs/view/4412749267</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Consultant (m/f/d) - Financial Services</t>
+          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Simon-Kucher</t>
+          <t>Carhartt WIP (Work In Progress)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46157</v>
+        <v>46153</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -2219,7 +2219,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/simon-kucher</t>
+          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2241,7 +2241,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>li-4411456773</t>
+          <t>li-4411718887</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411456773</t>
+          <t>https://www.linkedin.com/jobs/view/4411718887</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -2290,7 +2290,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -2312,7 +2312,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>li-4416856371</t>
+          <t>li-4409247899</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2322,27 +2322,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416856371</t>
+          <t>https://www.linkedin.com/jobs/view/4409247899</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Filialleiter:in / Store Manager 100% - Basel</t>
+          <t>Content Specialist</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Veloplus AG</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46168</v>
+        <v>46149</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -2361,7 +2361,7 @@
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/veloplus-ag</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -2383,7 +2383,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>li-4359225027</t>
+          <t>li-4398599784</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2393,23 +2393,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359225027</t>
+          <t>https://www.linkedin.com/jobs/view/4398599784</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Manager</t>
+          <t>Vice President, Business Manager</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Revolut</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>AMETEK</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Reinach, Basel-Country, Switzerland</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n">
-        <v>46166</v>
+        <v>46162</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -2428,7 +2432,7 @@
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/revolut</t>
+          <t>https://www.linkedin.com/company/ametek</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -2450,7 +2454,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>li-4398599784</t>
+          <t>li-4411990173</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2460,27 +2464,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4398599784</t>
+          <t>https://www.linkedin.com/jobs/view/4411990173</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Vice President, Business Manager</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AMETEK</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Reinach, Basel-Country, Switzerland</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46162</v>
+        <v>46151</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -2499,7 +2503,7 @@
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ametek</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -2521,7 +2525,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>li-4421813206</t>
+          <t>li-4410009795</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2531,26 +2535,28 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4421813206</t>
+          <t>https://www.linkedin.com/jobs/view/4410009795</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Business / Senior Consultant</t>
+          <t>Responsable Production H/F</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>MAK Consulting AG</t>
+          <t>L’univers NOZ</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Zollikofen, Berne, Switzerland</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>Strasbourg, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>46167</v>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -2568,7 +2574,7 @@
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mak-consulting-ag</t>
+          <t>https://fr.linkedin.com/company/lunivers-noz</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -2590,7 +2596,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>li-4414586149</t>
+          <t>li-4411456773</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2600,7 +2606,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414586149</t>
+          <t>https://www.linkedin.com/jobs/view/4411456773</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -2620,7 +2626,7 @@
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46156</v>
+        <v>46149</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -2661,7 +2667,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>li-4411984255</t>
+          <t>li-4412263197</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2671,27 +2677,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411984255</t>
+          <t>https://www.linkedin.com/jobs/view/4412263197</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>SThree</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46151</v>
+        <v>46160</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -2710,7 +2716,7 @@
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W31" t="inlineStr"/>
@@ -2732,7 +2738,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>li-4410039212</t>
+          <t>li-4412289349</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2742,23 +2748,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410039212</t>
+          <t>https://www.linkedin.com/jobs/view/4412289349</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Country Manager Germany</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>DeWarmte</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>SThree</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="n">
-        <v>46146</v>
+        <v>46160</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -2777,7 +2787,7 @@
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/dewarmte</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W32" t="inlineStr"/>
@@ -2799,7 +2809,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>li-4412263197</t>
+          <t>li-4410012963</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2809,18 +2819,18 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412263197</t>
+          <t>https://www.linkedin.com/jobs/view/4410012963</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Senior Associate - Consulting</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>VIVALDI_</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2829,7 +2839,7 @@
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46160</v>
+        <v>46121</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -2848,7 +2858,7 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://www.linkedin.com/company/vivaldi-group</t>
         </is>
       </c>
       <c r="W33" t="inlineStr"/>
@@ -2870,7 +2880,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>li-4412289349</t>
+          <t>li-4389002832</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2880,27 +2890,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412289349</t>
+          <t>https://www.linkedin.com/jobs/view/4389002832</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Management Consultant (d/f/m), DHL Consulting Europe</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>DHL</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46160</v>
+        <v>46105</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -2919,7 +2929,7 @@
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://de.linkedin.com/company/dhl</t>
         </is>
       </c>
       <c r="W34" t="inlineStr"/>
@@ -2941,7 +2951,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>li-4410012963</t>
+          <t>li-4048085587</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2951,18 +2961,18 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410012963</t>
+          <t>https://www.linkedin.com/jobs/view/4048085587</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Associate - Consulting</t>
+          <t>(Junior) Consultant (w/m/d) Banking &amp; Financial Institutions</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VIVALDI_</t>
+          <t>Horváth</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2971,7 +2981,7 @@
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>46121</v>
+        <v>45580</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
@@ -2990,7 +3000,7 @@
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/vivaldi-group</t>
+          <t>https://de.linkedin.com/company/horvathpartners</t>
         </is>
       </c>
       <c r="W35" t="inlineStr"/>
@@ -3012,7 +3022,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>li-4389002832</t>
+          <t>li-4407754531</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3022,27 +3032,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4389002832</t>
+          <t>https://www.linkedin.com/jobs/view/4407754531</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Management Consultant (d/f/m), DHL Consulting Europe</t>
+          <t>Supply Chain Lead (gn) bei SAMSUNG</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>DHL</t>
+          <t>Grafton Recruitment</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>46105</v>
+        <v>46164</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -3061,7 +3071,7 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/dhl</t>
+          <t>https://it.linkedin.com/company/grafton-recruitment</t>
         </is>
       </c>
       <c r="W36" t="inlineStr"/>
@@ -3083,7 +3093,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>li-4048085587</t>
+          <t>li-4412263197</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3093,18 +3103,18 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4048085587</t>
+          <t>https://www.linkedin.com/jobs/view/4412263197</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>(Junior) Consultant (w/m/d) Banking &amp; Financial Institutions</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Horváth</t>
+          <t>SThree</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3113,7 +3123,7 @@
         </is>
       </c>
       <c r="H37" s="2" t="n">
-        <v>45580</v>
+        <v>46160</v>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
@@ -3132,7 +3142,7 @@
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/horvathpartners</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W37" t="inlineStr"/>
@@ -3154,7 +3164,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>li-4384316600</t>
+          <t>li-4412289349</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3164,27 +3174,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4384316600</t>
+          <t>https://www.linkedin.com/jobs/view/4412289349</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sales Area Manager Nürnberg Würzburg (w_m_d)</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Barilla Group</t>
+          <t>SThree</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -3203,7 +3213,7 @@
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/barilla-group</t>
+          <t>https://uk.linkedin.com/company/sthree-plc</t>
         </is>
       </c>
       <c r="W38" t="inlineStr"/>
@@ -3225,7 +3235,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>li-4413931472</t>
+          <t>li-4416248930</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3235,18 +3245,18 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413931472</t>
+          <t>https://www.linkedin.com/jobs/view/4416248930</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Store Manager (m/w/d), Emporio Armani Düsseldorf</t>
+          <t>Recruitment Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Giorgio Armani</t>
+          <t>Ostendorf Consulting</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3255,7 +3265,7 @@
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46155</v>
+        <v>46160</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -3274,7 +3284,7 @@
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/giorgio-armani</t>
+          <t>https://de.linkedin.com/company/ostendorf-consulting</t>
         </is>
       </c>
       <c r="W39" t="inlineStr"/>
@@ -3296,7 +3306,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>li-4411814591</t>
+          <t>li-4409342469</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3306,27 +3316,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411814591</t>
+          <t>https://www.linkedin.com/jobs/view/4409342469</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>General Manager (STARS)*</t>
+          <t>Customer Onboarding Specialist</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tristar Hotels</t>
+          <t>eviivo</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Monheim, North Rhine-Westphalia, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>46149</v>
+        <v>46147</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -3345,7 +3355,7 @@
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/tristarhotels</t>
+          <t>https://uk.linkedin.com/company/eviivo</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
@@ -3367,7 +3377,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>li-4379922140</t>
+          <t>li-4411718887</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3377,27 +3387,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4379922140</t>
+          <t>https://www.linkedin.com/jobs/view/4411718887</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Area Manager - Cologne (m/f/d)</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>LAP Coffee</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>46083</v>
+        <v>46150</v>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
@@ -3416,7 +3426,7 @@
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/lap-coffee</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W41" t="inlineStr"/>
@@ -3438,7 +3448,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>li-4411990173</t>
+          <t>li-4404786229</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3448,27 +3458,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411990173</t>
+          <t>https://www.linkedin.com/jobs/view/4404786229</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Fraunhofer IAF</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>46151</v>
+        <v>46135</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -3487,7 +3497,7 @@
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
         </is>
       </c>
       <c r="W42" t="inlineStr"/>
@@ -3509,7 +3519,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>li-4407754531</t>
+          <t>li-4414586149</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3519,27 +3529,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407754531</t>
+          <t>https://www.linkedin.com/jobs/view/4414586149</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Supply Chain Lead (gn) bei SAMSUNG</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Grafton Recruitment</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Colmar, Grand Est, France</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>46164</v>
+        <v>46156</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -3558,7 +3568,7 @@
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/grafton-recruitment</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W43" t="inlineStr"/>
@@ -3580,7 +3590,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>li-4412263197</t>
+          <t>li-4411991147</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3590,27 +3600,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412263197</t>
+          <t>https://www.linkedin.com/jobs/view/4411991147</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>46160</v>
+        <v>46151</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -3629,7 +3639,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W44" t="inlineStr"/>
@@ -3651,7 +3661,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>li-4412289349</t>
+          <t>li-4411984255</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3661,27 +3671,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412289349</t>
+          <t>https://www.linkedin.com/jobs/view/4411984255</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>46160</v>
+        <v>46151</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -3700,7 +3710,7 @@
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W45" t="inlineStr"/>
@@ -3722,7 +3732,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>li-4416248930</t>
+          <t>li-4386750509</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3732,27 +3742,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416248930</t>
+          <t>https://www.linkedin.com/jobs/view/4386750509</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Spontanbewerbung</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Ostendorf Consulting</t>
+          <t>INFORS HT</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Bottmingen, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H46" s="2" t="n">
-        <v>46160</v>
+        <v>46098</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -3771,7 +3781,7 @@
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/ostendorf-consulting</t>
+          <t>https://ch.linkedin.com/company/inforsht</t>
         </is>
       </c>
       <c r="W46" t="inlineStr"/>
@@ -3790,361 +3800,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>li-4409342469</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4409342469</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Customer Onboarding Specialist</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>eviivo</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="n">
-        <v>46147</v>
-      </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="b">
-        <v>0</v>
-      </c>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
-      <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>https://uk.linkedin.com/company/eviivo</t>
-        </is>
-      </c>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
-      <c r="Y47" t="inlineStr"/>
-      <c r="Z47" t="inlineStr"/>
-      <c r="AA47" t="inlineStr"/>
-      <c r="AB47" t="inlineStr"/>
-      <c r="AC47" t="inlineStr"/>
-      <c r="AD47" t="inlineStr"/>
-      <c r="AE47" t="inlineStr"/>
-      <c r="AF47" t="inlineStr"/>
-      <c r="AG47" t="inlineStr"/>
-      <c r="AH47" t="inlineStr"/>
-      <c r="AI47" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>li-4411718887</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Business &amp; Customer Data Analyst</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>MCH Group</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Basel, Switzerland</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="n">
-        <v>46150</v>
-      </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="b">
-        <v>0</v>
-      </c>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
-      <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
-        </is>
-      </c>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
-      <c r="Y48" t="inlineStr"/>
-      <c r="Z48" t="inlineStr"/>
-      <c r="AA48" t="inlineStr"/>
-      <c r="AB48" t="inlineStr"/>
-      <c r="AC48" t="inlineStr"/>
-      <c r="AD48" t="inlineStr"/>
-      <c r="AE48" t="inlineStr"/>
-      <c r="AF48" t="inlineStr"/>
-      <c r="AG48" t="inlineStr"/>
-      <c r="AH48" t="inlineStr"/>
-      <c r="AI48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>li-4404786229</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4404786229</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Fraunhofer IAF</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="b">
-        <v>0</v>
-      </c>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
-      <c r="T49" t="inlineStr"/>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
-        </is>
-      </c>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
-      <c r="Y49" t="inlineStr"/>
-      <c r="Z49" t="inlineStr"/>
-      <c r="AA49" t="inlineStr"/>
-      <c r="AB49" t="inlineStr"/>
-      <c r="AC49" t="inlineStr"/>
-      <c r="AD49" t="inlineStr"/>
-      <c r="AE49" t="inlineStr"/>
-      <c r="AF49" t="inlineStr"/>
-      <c r="AG49" t="inlineStr"/>
-      <c r="AH49" t="inlineStr"/>
-      <c r="AI49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>li-4411991147</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4411991147</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Strasbourg, Grand Est, France</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="n">
-        <v>46151</v>
-      </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="b">
-        <v>0</v>
-      </c>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
-      <c r="T50" t="inlineStr"/>
-      <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
-      <c r="Z50" t="inlineStr"/>
-      <c r="AA50" t="inlineStr"/>
-      <c r="AB50" t="inlineStr"/>
-      <c r="AC50" t="inlineStr"/>
-      <c r="AD50" t="inlineStr"/>
-      <c r="AE50" t="inlineStr"/>
-      <c r="AF50" t="inlineStr"/>
-      <c r="AG50" t="inlineStr"/>
-      <c r="AH50" t="inlineStr"/>
-      <c r="AI50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>li-4386750509</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4386750509</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Spontanbewerbung</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>INFORS HT</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Bottmingen, Basel-Country, Switzerland</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="n">
-        <v>46098</v>
-      </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="b">
-        <v>0</v>
-      </c>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
-      <c r="T51" t="inlineStr"/>
-      <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>https://ch.linkedin.com/company/inforsht</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
-      <c r="Z51" t="inlineStr"/>
-      <c r="AA51" t="inlineStr"/>
-      <c r="AB51" t="inlineStr"/>
-      <c r="AC51" t="inlineStr"/>
-      <c r="AD51" t="inlineStr"/>
-      <c r="AE51" t="inlineStr"/>
-      <c r="AF51" t="inlineStr"/>
-      <c r="AG51" t="inlineStr"/>
-      <c r="AH51" t="inlineStr"/>
-      <c r="AI51" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Job Report Fri Jun  5 02:35:26 UTC 2026
</commit_message>
<xml_diff>
--- a/Latest_Job_Report.xlsx
+++ b/Latest_Job_Report.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI46"/>
+  <dimension ref="A1:AI61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -683,7 +683,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>li-4404056876</t>
+          <t>li-4417524508</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -693,27 +693,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404056876</t>
+          <t>https://www.linkedin.com/jobs/view/4417524508</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>AIML - Research Scientist, Health</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The IN Group</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46170</v>
+        <v>46165</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -732,7 +732,7 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/we-are-tig</t>
+          <t>https://www.linkedin.com/company/apple</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -754,7 +754,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>li-4413525792</t>
+          <t>li-4141647343</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -764,23 +764,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413525792</t>
+          <t>https://www.linkedin.com/jobs/view/4141647343</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Market Researcher</t>
+          <t>Research Scientist (Zurich Location)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Xiaomi Technology</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>RAI Institute</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="n">
-        <v>46154</v>
+        <v>45692</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -799,7 +803,7 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
+          <t>https://www.linkedin.com/company/rai-inst</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -821,7 +825,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>li-4407397044</t>
+          <t>li-4404056876</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -831,27 +835,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407397044</t>
+          <t>https://www.linkedin.com/jobs/view/4404056876</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Deutsches Diabetes-Zentrum</t>
+          <t>The IN Group</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46142</v>
+        <v>46170</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -870,7 +874,7 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
+          <t>https://uk.linkedin.com/company/we-are-tig</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -892,7 +896,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>li-4257970631</t>
+          <t>li-4413434561</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -902,27 +906,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4257970631</t>
+          <t>https://www.linkedin.com/jobs/view/4413434561</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
+          <t>Research Assistant for Physics Laboratory (50%)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>WHU Entrepreneurship Roundtable</t>
+          <t>University of Applied Sciences and Arts Northwestern Switzerland FHNW</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Vallendar, Rhineland-Palatinate, Germany</t>
+          <t>Windisch, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>45813</v>
+        <v>46154</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -941,7 +945,7 @@
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
+          <t>https://ch.linkedin.com/school/fachhochschule-nordwestschweiz-fhnw/</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -963,7 +967,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>li-4418110532</t>
+          <t>li-4414163533</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -973,27 +977,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4418110532</t>
+          <t>https://www.linkedin.com/jobs/view/4414163533</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Medical Researcher (m/w/d)</t>
+          <t>AIML - Machine Learning Research, Multimodal Foundation Models</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Deutsches Promotionszentrum</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46164</v>
+        <v>46155</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -1012,7 +1016,7 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
+          <t>https://www.linkedin.com/company/apple</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1034,7 +1038,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>li-4404056876</t>
+          <t>li-4387421660</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1044,27 +1048,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404056876</t>
+          <t>https://www.linkedin.com/jobs/view/4387421660</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Research Scientist, Gemini Safety</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>The IN Group</t>
+          <t>Google DeepMind</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46170</v>
+        <v>46164</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1083,7 +1087,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/we-are-tig</t>
+          <t>https://uk.linkedin.com/company/googledeepmind</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1105,7 +1109,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4415995749</t>
+          <t>li-4404480766</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1115,18 +1119,18 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4415995749</t>
+          <t>https://www.linkedin.com/jobs/view/4404480766</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Investment Research Analyst</t>
+          <t>Research Scientist, 3D Computer Vision</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1134,9 +1138,7 @@
           <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
-        <v>46162</v>
-      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1154,7 +1156,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://www.linkedin.com/company/nvidia</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1176,7 +1178,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4414173590</t>
+          <t>li-4418110532</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1186,27 +1188,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414173590</t>
+          <t>https://www.linkedin.com/jobs/view/4418110532</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Investment Research Analyst | Upto $100/hr</t>
+          <t>Medical Researcher (m/w/d)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>Deutsches Promotionszentrum</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46155</v>
+        <v>46164</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1225,7 +1227,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1247,7 +1249,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4410472579</t>
+          <t>li-4257970631</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1257,27 +1259,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410472579</t>
+          <t>https://www.linkedin.com/jobs/view/4257970631</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Quantitative Researcher</t>
+          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>STS Digital Group</t>
+          <t>WHU Entrepreneurship Roundtable</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Vallendar, Rhineland-Palatinate, Germany</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46149</v>
+        <v>45813</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1296,7 +1298,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sts-digital-group</t>
+          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1318,7 +1320,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4413434561</t>
+          <t>li-4407397044</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1328,27 +1330,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413434561</t>
+          <t>https://www.linkedin.com/jobs/view/4407397044</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Research Assistant for Physics Laboratory (50%)</t>
+          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>University of Applied Sciences and Arts Northwestern Switzerland FHNW</t>
+          <t>Deutsches Diabetes-Zentrum</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Windisch, Aargau, Switzerland</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46154</v>
+        <v>46142</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1367,7 +1369,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/school/fachhochschule-nordwestschweiz-fhnw/</t>
+          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1389,7 +1391,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>li-4377188248</t>
+          <t>li-4413525792</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1399,27 +1401,23 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4377188248</t>
+          <t>https://www.linkedin.com/jobs/view/4413525792</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Working Student - Executive Researcher 50% hybrid (m/f)</t>
+          <t>Senior Market Researcher</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Franke Group</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Aarburg, Aargau, Switzerland</t>
-        </is>
-      </c>
+          <t>Xiaomi Technology</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" s="2" t="n">
-        <v>46162</v>
+        <v>46154</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1438,7 +1436,7 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/franke-group</t>
+          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -1460,7 +1458,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>li-4409306761</t>
+          <t>li-4414586149</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1470,27 +1468,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409306761</t>
+          <t>https://www.linkedin.com/jobs/view/4414586149</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Country Manager Belgium and Luxembourg (BeLux-based) 🇧🇪🇱🇺</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Chargemap</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Colmar, Grand Est, France</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46147</v>
+        <v>46156</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1509,7 +1507,7 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/chargemap</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -1531,7 +1529,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>li-4408692266</t>
+          <t>li-4335125314</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1541,27 +1539,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4408692266</t>
+          <t>https://www.linkedin.com/jobs/view/4335125314</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Country Sales Manager Schweiz (mwd)</t>
+          <t>Consultant - Operations Excellence Program</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>CCR Commercial Refrigeration</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pratteln, Basel-Country, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46146</v>
+        <v>46166</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1580,7 +1578,7 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -1602,7 +1600,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>li-4335125314</t>
+          <t>li-4423364166</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1612,28 +1610,26 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4335125314</t>
+          <t>https://www.linkedin.com/jobs/view/4423364166</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Consultant - Operations Excellence Program</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>46166</v>
-      </c>
+          <t>Colmar, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -1651,7 +1647,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -1673,7 +1669,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>li-4404786229</t>
+          <t>li-4416485748</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1683,27 +1679,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404786229</t>
+          <t>https://www.linkedin.com/jobs/view/4416485748</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
+          <t>Drug Safety Case Manager</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Fraunhofer IAF</t>
+          <t>Flexsis</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Allschwil, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46135</v>
+        <v>46161</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1722,7 +1718,7 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
+          <t>https://ch.linkedin.com/company/flexsisch</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -1744,7 +1740,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>li-4413366651</t>
+          <t>li-4417604986</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1754,27 +1750,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413366651</t>
+          <t>https://www.linkedin.com/jobs/view/4417604986</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assistant General Manager / Assistenz der Hoteldirektion (m/w/d)</t>
+          <t>Facility Coordinator (a) 80%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hotel Am Rathaus Freibug</t>
+          <t>JYSK</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Zofingen, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46162</v>
+        <v>46170</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1793,7 +1789,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/hotel-am-rathaus-freibug</t>
+          <t>https://dk.linkedin.com/company/jysk</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -1815,7 +1811,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>li-4335254607</t>
+          <t>li-4411718887</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1825,27 +1821,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4335254607</t>
+          <t>https://www.linkedin.com/jobs/view/4411718887</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Consultant - Procurement</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46166</v>
+        <v>46150</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1864,7 +1860,7 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -1886,7 +1882,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>li-4417067089</t>
+          <t>li-4320219168</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1896,18 +1892,18 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4417067089</t>
+          <t>https://www.linkedin.com/jobs/view/4320219168</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Consultant / Manager Strategy Consulting</t>
+          <t>(Senior) Consultant - Business Consulting - Finance</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>LEAP PARTNERS</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1916,7 +1912,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46162</v>
+        <v>46157</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1935,7 +1931,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/leap-partners</t>
+          <t>https://uk.linkedin.com/company/ernstandyoung</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -1957,7 +1953,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>li-4416102577</t>
+          <t>li-4335254607</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1967,18 +1963,18 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416102577</t>
+          <t>https://www.linkedin.com/jobs/view/4335254607</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Management Consultant</t>
+          <t>Consultant - Procurement</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1987,7 +1983,7 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46162</v>
+        <v>46166</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -2006,7 +2002,7 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2028,7 +2024,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>li-4414574747</t>
+          <t>li-4409306761</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2038,27 +2034,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414574747</t>
+          <t>https://www.linkedin.com/jobs/view/4409306761</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Country Manager Belgium and Luxembourg (BeLux-based) 🇧🇪🇱🇺</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Chargemap</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Belfort, Bourgogne-Franche-Comté, France</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46156</v>
+        <v>46147</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -2077,7 +2073,7 @@
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://fr.linkedin.com/company/chargemap</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2099,7 +2095,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>li-4416485748</t>
+          <t>li-4414574747</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2109,27 +2105,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416485748</t>
+          <t>https://www.linkedin.com/jobs/view/4414574747</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Drug Safety Case Manager</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Flexsis</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Allschwil, Basel-Country, Switzerland</t>
+          <t>Belfort, Bourgogne-Franche-Comté, France</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46161</v>
+        <v>46156</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -2148,7 +2144,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/flexsisch</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2170,7 +2166,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>li-4412749267</t>
+          <t>li-4423364166</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2180,28 +2176,26 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412749267</t>
+          <t>https://www.linkedin.com/jobs/view/4423364166</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Carhartt WIP (Work In Progress)</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>46153</v>
-      </c>
+          <t>Colmar, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
@@ -2219,7 +2213,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2241,7 +2235,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4422364081</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2251,27 +2245,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4422364081</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Responsable de magasin  H/F</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>BLACKSTORE France</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Saint-Louis, Grand Est, France</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46150</v>
+        <v>46175</v>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -2290,7 +2284,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://fr.linkedin.com/company/blackstore</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -2312,7 +2306,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>li-4409247899</t>
+          <t>li-4416856371</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2322,27 +2316,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409247899</t>
+          <t>https://www.linkedin.com/jobs/view/4416856371</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Content Specialist</t>
+          <t>Filialleiter:in / Store Manager 100% - Basel</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>Veloplus AG</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46149</v>
+        <v>46168</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -2361,7 +2355,7 @@
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://ch.linkedin.com/company/veloplus-ag</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -2383,7 +2377,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>li-4398599784</t>
+          <t>li-4359225027</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2393,27 +2387,23 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4398599784</t>
+          <t>https://www.linkedin.com/jobs/view/4359225027</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Vice President, Business Manager</t>
+          <t>Strategy &amp; Operations Manager</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>AMETEK</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Reinach, Basel-Country, Switzerland</t>
-        </is>
-      </c>
+          <t>Revolut</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" s="2" t="n">
-        <v>46162</v>
+        <v>46166</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -2432,7 +2422,7 @@
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ametek</t>
+          <t>https://uk.linkedin.com/company/revolut</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -2454,7 +2444,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>li-4411990173</t>
+          <t>li-4408692266</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2464,27 +2454,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411990173</t>
+          <t>https://www.linkedin.com/jobs/view/4408692266</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Country Sales Manager Schweiz (mwd)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>CCR Commercial Refrigeration</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Pratteln, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46151</v>
+        <v>46146</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -2503,7 +2493,7 @@
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -2525,7 +2515,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>li-4410009795</t>
+          <t>li-4392923773</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2535,27 +2525,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410009795</t>
+          <t>https://www.linkedin.com/jobs/view/4392923773</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Responsable Production H/F</t>
+          <t>Manager/in Operations (m/w/d)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>L’univers NOZ</t>
+          <t>Thommen Group</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Aarwangen, Berne, Switzerland</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46167</v>
+        <v>46111</v>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -2574,7 +2564,7 @@
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/lunivers-noz</t>
+          <t>https://ch.linkedin.com/company/thommengroup</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -2596,7 +2586,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>li-4411456773</t>
+          <t>li-4416485748</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2606,27 +2596,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411456773</t>
+          <t>https://www.linkedin.com/jobs/view/4416485748</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Drug Safety Case Manager</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Flexsis</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Allschwil, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46149</v>
+        <v>46161</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -2645,7 +2635,7 @@
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://ch.linkedin.com/company/flexsisch</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
@@ -2667,7 +2657,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>li-4412263197</t>
+          <t>li-4412749267</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2677,27 +2667,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412263197</t>
+          <t>https://www.linkedin.com/jobs/view/4412749267</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>Carhartt WIP (Work In Progress)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -2716,7 +2706,7 @@
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
         </is>
       </c>
       <c r="W31" t="inlineStr"/>
@@ -2738,7 +2728,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>li-4412289349</t>
+          <t>li-4411718887</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2748,27 +2738,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412289349</t>
+          <t>https://www.linkedin.com/jobs/view/4411718887</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46160</v>
+        <v>46150</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -2787,7 +2777,7 @@
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W32" t="inlineStr"/>
@@ -2809,7 +2799,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>li-4410012963</t>
+          <t>li-4409247899</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2819,27 +2809,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410012963</t>
+          <t>https://www.linkedin.com/jobs/view/4409247899</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Senior Associate - Consulting</t>
+          <t>Content Specialist</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>VIVALDI_</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46121</v>
+        <v>46149</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -2858,7 +2848,7 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/vivaldi-group</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W33" t="inlineStr"/>
@@ -2880,7 +2870,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>li-4389002832</t>
+          <t>li-4408692266</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2890,27 +2880,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4389002832</t>
+          <t>https://www.linkedin.com/jobs/view/4408692266</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Management Consultant (d/f/m), DHL Consulting Europe</t>
+          <t>Country Sales Manager Schweiz (mwd)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>DHL</t>
+          <t>CCR Commercial Refrigeration</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Pratteln, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46105</v>
+        <v>46146</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -2929,7 +2919,7 @@
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/dhl</t>
+          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
         </is>
       </c>
       <c r="W34" t="inlineStr"/>
@@ -2951,7 +2941,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>li-4048085587</t>
+          <t>li-4410009795</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2961,27 +2951,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4048085587</t>
+          <t>https://www.linkedin.com/jobs/view/4410009795</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>(Junior) Consultant (w/m/d) Banking &amp; Financial Institutions</t>
+          <t>Responsable Production H/F</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Horváth</t>
+          <t>L’univers NOZ</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>45580</v>
+        <v>46167</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
@@ -3000,7 +2990,7 @@
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/horvathpartners</t>
+          <t>https://fr.linkedin.com/company/lunivers-noz</t>
         </is>
       </c>
       <c r="W35" t="inlineStr"/>
@@ -3022,7 +3012,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>li-4407754531</t>
+          <t>li-4398599784</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3032,27 +3022,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407754531</t>
+          <t>https://www.linkedin.com/jobs/view/4398599784</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Supply Chain Lead (gn) bei SAMSUNG</t>
+          <t>Vice President, Business Manager</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Grafton Recruitment</t>
+          <t>AMETEK</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Reinach, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>46164</v>
+        <v>46162</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -3071,7 +3061,7 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/grafton-recruitment</t>
+          <t>https://www.linkedin.com/company/ametek</t>
         </is>
       </c>
       <c r="W36" t="inlineStr"/>
@@ -3093,7 +3083,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>li-4412263197</t>
+          <t>li-4413366651</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3103,27 +3093,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412263197</t>
+          <t>https://www.linkedin.com/jobs/view/4413366651</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Assistant General Manager / Assistenz der Hoteldirektion (m/w/d)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>Hotel Am Rathaus Freibug</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
-        <v>46160</v>
+        <v>46162</v>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
@@ -3142,7 +3132,7 @@
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://www.linkedin.com/company/hotel-am-rathaus-freibug</t>
         </is>
       </c>
       <c r="W37" t="inlineStr"/>
@@ -3164,7 +3154,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>li-4412289349</t>
+          <t>li-4420147175</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3174,18 +3164,18 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412289349</t>
+          <t>https://www.linkedin.com/jobs/view/4420147175</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>SThree</t>
+          <t>Bain &amp; Company</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3194,7 +3184,7 @@
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>46160</v>
+        <v>46176</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -3213,7 +3203,7 @@
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/sthree-plc</t>
+          <t>https://www.linkedin.com/company/bain-and-company</t>
         </is>
       </c>
       <c r="W38" t="inlineStr"/>
@@ -3235,7 +3225,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>li-4416248930</t>
+          <t>li-4301586122</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3245,18 +3235,18 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416248930</t>
+          <t>https://www.linkedin.com/jobs/view/4301586122</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Recruitment Consultant (m/w/d)</t>
+          <t>Experienced Consultant - Capital Excellence</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Ostendorf Consulting</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3265,7 +3255,7 @@
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46160</v>
+        <v>46176</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -3284,7 +3274,7 @@
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/ostendorf-consulting</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W39" t="inlineStr"/>
@@ -3306,7 +3296,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>li-4409342469</t>
+          <t>li-4301569738</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3316,27 +3306,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409342469</t>
+          <t>https://www.linkedin.com/jobs/view/4301569738</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Customer Onboarding Specialist</t>
+          <t>Experienced Consultant - Capital Excellence</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>eviivo</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>46147</v>
+        <v>46173</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -3355,7 +3345,7 @@
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/eviivo</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
@@ -3377,7 +3367,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4266954854</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3387,27 +3377,23 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4266954854</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Experienced Consultant (Düsseldorf)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>MCH Group</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Basel, Switzerland</t>
-        </is>
-      </c>
+          <t>OC&amp;C Strategy Consultants</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" s="2" t="n">
-        <v>46150</v>
+        <v>46161</v>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
@@ -3426,7 +3412,7 @@
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://uk.linkedin.com/company/oc&amp;c-strategy-consultants</t>
         </is>
       </c>
       <c r="W41" t="inlineStr"/>
@@ -3448,7 +3434,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>li-4404786229</t>
+          <t>li-4371968232</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3458,27 +3444,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404786229</t>
+          <t>https://www.linkedin.com/jobs/view/4371968232</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
+          <t>Consultant (w/m/d) Public Sector</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Fraunhofer IAF</t>
+          <t>Horváth</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>46135</v>
+        <v>46070</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -3497,7 +3483,7 @@
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
+          <t>https://de.linkedin.com/company/horvathpartners</t>
         </is>
       </c>
       <c r="W42" t="inlineStr"/>
@@ -3519,7 +3505,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>li-4414586149</t>
+          <t>li-4384316600</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3529,27 +3515,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414586149</t>
+          <t>https://www.linkedin.com/jobs/view/4384316600</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Sales Area Manager Nürnberg Würzburg (w_m_d)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Barilla Group</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -3568,7 +3554,7 @@
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://it.linkedin.com/company/barilla-group</t>
         </is>
       </c>
       <c r="W43" t="inlineStr"/>
@@ -3590,7 +3576,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>li-4411991147</t>
+          <t>li-4413931472</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3600,27 +3586,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411991147</t>
+          <t>https://www.linkedin.com/jobs/view/4413931472</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Store Manager (m/w/d), Emporio Armani Düsseldorf</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Giorgio Armani</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>46151</v>
+        <v>46155</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -3639,7 +3625,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://it.linkedin.com/company/giorgio-armani</t>
         </is>
       </c>
       <c r="W44" t="inlineStr"/>
@@ -3661,7 +3647,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>li-4411984255</t>
+          <t>li-4412707731</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3671,27 +3657,23 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411984255</t>
+          <t>https://www.linkedin.com/jobs/view/4412707731</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Retail Operation Manager</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Strasbourg, Grand Est, France</t>
-        </is>
-      </c>
+          <t>Anker Innovations</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" s="2" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -3710,7 +3692,7 @@
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://www.linkedin.com/company/ankerinnovations</t>
         </is>
       </c>
       <c r="W45" t="inlineStr"/>
@@ -3732,7 +3714,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>li-4386750509</t>
+          <t>li-4410039212</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3742,27 +3724,23 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386750509</t>
+          <t>https://www.linkedin.com/jobs/view/4410039212</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Spontanbewerbung</t>
+          <t>Country Manager Germany</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>INFORS HT</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Bottmingen, Basel-Country, Switzerland</t>
-        </is>
-      </c>
+          <t>DeWarmte</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" s="2" t="n">
-        <v>46098</v>
+        <v>46146</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -3781,7 +3759,7 @@
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/inforsht</t>
+          <t>https://nl.linkedin.com/company/dewarmte</t>
         </is>
       </c>
       <c r="W46" t="inlineStr"/>
@@ -3800,6 +3778,1063 @@
         <v>0</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>li-4379922140</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4379922140</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Area Manager - Cologne (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>LAP Coffee</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="b">
+        <v>0</v>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/lap-coffee</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
+      <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr"/>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr"/>
+      <c r="AI47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>li-4423985038</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4423985038</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BaSE Specialist (m/w/d)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="b">
+        <v>0</v>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/ups</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
+      <c r="AD48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr"/>
+      <c r="AF48" t="inlineStr"/>
+      <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr"/>
+      <c r="AI48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>li-4421807992</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4421807992</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Revisor Specialist - Penny International (m/w/d)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PENNY International (REWE Group)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="b">
+        <v>0</v>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/penny-international-rewe-group</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr"/>
+      <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr"/>
+      <c r="AI49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>li-4422122505</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4422122505</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Senior Specialist BCM Production (m/w/d)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Vaillant Deutschland</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Remscheid, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="b">
+        <v>0</v>
+      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/vaillantdeutschland</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr"/>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>li-4419053552</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4419053552</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Order Management Specialist</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Octave</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="b">
+        <v>0</v>
+      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/octaveintelligence</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="inlineStr"/>
+      <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr"/>
+      <c r="AI51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>li-4416894948</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4416894948</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Spezialist (m/w/d) für Einlagensicherung</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Prüfungsverband deutscher Banken e.V.</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>46169</v>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="b">
+        <v>0</v>
+      </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/pruefungsverbanddeutscherbanken</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
+      <c r="AF52" t="inlineStr"/>
+      <c r="AG52" t="inlineStr"/>
+      <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>li-4419276665</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4419276665</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Senior Analyst:in</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Gi Group</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Basel, Switzerland</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="b">
+        <v>0</v>
+      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>https://it.linkedin.com/company/gi-group</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr"/>
+      <c r="AC53" t="inlineStr"/>
+      <c r="AD53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr"/>
+      <c r="AF53" t="inlineStr"/>
+      <c r="AG53" t="inlineStr"/>
+      <c r="AH53" t="inlineStr"/>
+      <c r="AI53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>li-4411718887</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Business &amp; Customer Data Analyst</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>MCH Group</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Basel, Switzerland</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>46150</v>
+      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="b">
+        <v>0</v>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr"/>
+      <c r="AD54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr"/>
+      <c r="AF54" t="inlineStr"/>
+      <c r="AG54" t="inlineStr"/>
+      <c r="AH54" t="inlineStr"/>
+      <c r="AI54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>li-4404786229</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4404786229</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Fraunhofer IAF</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="b">
+        <v>0</v>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr"/>
+      <c r="AD55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr"/>
+      <c r="AF55" t="inlineStr"/>
+      <c r="AG55" t="inlineStr"/>
+      <c r="AH55" t="inlineStr"/>
+      <c r="AI55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>li-4414586149</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4414586149</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Colmar, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>46156</v>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="b">
+        <v>0</v>
+      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr"/>
+      <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr"/>
+      <c r="AD56" t="inlineStr"/>
+      <c r="AE56" t="inlineStr"/>
+      <c r="AF56" t="inlineStr"/>
+      <c r="AG56" t="inlineStr"/>
+      <c r="AH56" t="inlineStr"/>
+      <c r="AI56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>li-4423364166</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4423364166</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Colmar, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="b">
+        <v>0</v>
+      </c>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr"/>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
+      <c r="Z57" t="inlineStr"/>
+      <c r="AA57" t="inlineStr"/>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr"/>
+      <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr"/>
+      <c r="AG57" t="inlineStr"/>
+      <c r="AH57" t="inlineStr"/>
+      <c r="AI57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>li-4423350822</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4423350822</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Strasbourg, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="b">
+        <v>0</v>
+      </c>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr"/>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr"/>
+      <c r="X58" t="inlineStr"/>
+      <c r="Y58" t="inlineStr"/>
+      <c r="Z58" t="inlineStr"/>
+      <c r="AA58" t="inlineStr"/>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr"/>
+      <c r="AD58" t="inlineStr"/>
+      <c r="AE58" t="inlineStr"/>
+      <c r="AF58" t="inlineStr"/>
+      <c r="AG58" t="inlineStr"/>
+      <c r="AH58" t="inlineStr"/>
+      <c r="AI58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>li-4423362471</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4423362471</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Strasbourg, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="b">
+        <v>0</v>
+      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr"/>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr"/>
+      <c r="X59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr"/>
+      <c r="Z59" t="inlineStr"/>
+      <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr"/>
+      <c r="AD59" t="inlineStr"/>
+      <c r="AE59" t="inlineStr"/>
+      <c r="AF59" t="inlineStr"/>
+      <c r="AG59" t="inlineStr"/>
+      <c r="AH59" t="inlineStr"/>
+      <c r="AI59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>li-4423343998</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4423343998</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Strasbourg, Grand Est, France</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="b">
+        <v>0</v>
+      </c>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr"/>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr"/>
+      <c r="X60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr"/>
+      <c r="Z60" t="inlineStr"/>
+      <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr"/>
+      <c r="AD60" t="inlineStr"/>
+      <c r="AE60" t="inlineStr"/>
+      <c r="AF60" t="inlineStr"/>
+      <c r="AG60" t="inlineStr"/>
+      <c r="AH60" t="inlineStr"/>
+      <c r="AI60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>li-4386750509</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4386750509</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Spontanbewerbung</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>INFORS HT</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Bottmingen, Basel-Country, Switzerland</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="b">
+        <v>0</v>
+      </c>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>https://ch.linkedin.com/company/inforsht</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr"/>
+      <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr"/>
+      <c r="Z61" t="inlineStr"/>
+      <c r="AA61" t="inlineStr"/>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr"/>
+      <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
+      <c r="AF61" t="inlineStr"/>
+      <c r="AG61" t="inlineStr"/>
+      <c r="AH61" t="inlineStr"/>
+      <c r="AI61" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Job Report Tue Jun  9 02:11:49 UTC 2026
</commit_message>
<xml_diff>
--- a/Latest_Job_Report.xlsx
+++ b/Latest_Job_Report.xlsx
@@ -683,7 +683,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>li-4417524508</t>
+          <t>li-4404056876</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -693,27 +693,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4417524508</t>
+          <t>https://www.linkedin.com/jobs/view/4404056876</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AIML - Research Scientist, Health</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>The IN Group</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46165</v>
+        <v>46170</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -732,7 +732,7 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/apple</t>
+          <t>https://uk.linkedin.com/company/we-are-tig</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -754,7 +754,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>li-4141647343</t>
+          <t>li-4413525792</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -764,27 +764,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4141647343</t>
+          <t>https://www.linkedin.com/jobs/view/4413525792</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Research Scientist (Zurich Location)</t>
+          <t>Senior Market Researcher</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>RAI Institute</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Zurich, Zurich, Switzerland</t>
-        </is>
-      </c>
+          <t>Xiaomi Technology</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" s="2" t="n">
-        <v>45692</v>
+        <v>46154</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -803,7 +799,7 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/rai-inst</t>
+          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -825,7 +821,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>li-4404056876</t>
+          <t>li-4407397044</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -835,27 +831,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404056876</t>
+          <t>https://www.linkedin.com/jobs/view/4407397044</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>The IN Group</t>
+          <t>Deutsches Diabetes-Zentrum</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46170</v>
+        <v>46142</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -874,7 +870,7 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/we-are-tig</t>
+          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -896,7 +892,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>li-4413434561</t>
+          <t>li-4257970631</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -906,27 +902,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413434561</t>
+          <t>https://www.linkedin.com/jobs/view/4257970631</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Research Assistant for Physics Laboratory (50%)</t>
+          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>University of Applied Sciences and Arts Northwestern Switzerland FHNW</t>
+          <t>WHU Entrepreneurship Roundtable</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Windisch, Aargau, Switzerland</t>
+          <t>Vallendar, Rhineland-Palatinate, Germany</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46154</v>
+        <v>45813</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -945,7 +941,7 @@
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/school/fachhochschule-nordwestschweiz-fhnw/</t>
+          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -967,7 +963,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>li-4414163533</t>
+          <t>li-4418110532</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -977,27 +973,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414163533</t>
+          <t>https://www.linkedin.com/jobs/view/4418110532</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AIML - Machine Learning Research, Multimodal Foundation Models</t>
+          <t>Medical Researcher (m/w/d)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Deutsches Promotionszentrum</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46155</v>
+        <v>46164</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -1016,7 +1012,7 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/apple</t>
+          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1038,7 +1034,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>li-4387421660</t>
+          <t>li-4414173590</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1048,18 +1044,18 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387421660</t>
+          <t>https://www.linkedin.com/jobs/view/4414173590</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Research Scientist, Gemini Safety</t>
+          <t>Investment Research Analyst | Upto $100/hr</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Google DeepMind</t>
+          <t>Mercor</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1068,7 +1064,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46164</v>
+        <v>46155</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1087,7 +1083,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/googledeepmind</t>
+          <t>https://www.linkedin.com/company/mercor-ai</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1109,7 +1105,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4404480766</t>
+          <t>li-4407427079</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1119,26 +1115,28 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404480766</t>
+          <t>https://www.linkedin.com/jobs/view/4407427079</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Research Scientist, 3D Computer Vision</t>
+          <t>Research Scientist, Foundation Model</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Prior Labs</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>46139</v>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1156,7 +1154,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/nvidia</t>
+          <t>https://de.linkedin.com/company/prior-labs</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1178,7 +1176,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4418110532</t>
+          <t>li-4415995749</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1188,27 +1186,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4418110532</t>
+          <t>https://www.linkedin.com/jobs/view/4415995749</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Medical Researcher (m/w/d)</t>
+          <t>Investment Research Analyst</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Deutsches Promotionszentrum</t>
+          <t>Mercor</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46164</v>
+        <v>46162</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1227,7 +1225,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
+          <t>https://www.linkedin.com/company/mercor-ai</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1249,7 +1247,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4257970631</t>
+          <t>li-4417613007</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1259,27 +1257,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4257970631</t>
+          <t>https://www.linkedin.com/jobs/view/4417613007</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
+          <t>Research Associate - Chemistry</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>WHU Entrepreneurship Roundtable</t>
+          <t>UNSW</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Vallendar, Rhineland-Palatinate, Germany</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>45813</v>
+        <v>46170</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1298,7 +1296,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
+          <t>https://au.linkedin.com/school/unsw/</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1320,7 +1318,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4407397044</t>
+          <t>li-4386853728</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1330,27 +1328,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407397044</t>
+          <t>https://www.linkedin.com/jobs/view/4386853728</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
+          <t>Senior Network Specialist</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Deutsches Diabetes-Zentrum</t>
+          <t>Spektrum</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46142</v>
+        <v>46100</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1369,7 +1367,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
+          <t>https://es.linkedin.com/company/spektrumgrp</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1385,13 +1383,13 @@
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr"/>
       <c r="AI12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>li-4413525792</t>
+          <t>li-4380147309</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1401,23 +1399,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413525792</t>
+          <t>https://www.linkedin.com/jobs/view/4380147309</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Market Researcher</t>
+          <t>KONSTANZ - Kundenservice / Station Service Specialist (m/w/d)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Xiaomi Technology</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>roadsurfer</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Aach, Baden-Württemberg, Germany</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="n">
-        <v>46154</v>
+        <v>46084</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1436,7 +1438,7 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
+          <t>https://de.linkedin.com/company/roadsurfer-gmbh</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -1452,13 +1454,13 @@
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>li-4414586149</t>
+          <t>li-4386868249</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1468,27 +1470,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414586149</t>
+          <t>https://www.linkedin.com/jobs/view/4386868249</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Senior Continuous Service Improvement Specialist</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Spektrum</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46156</v>
+        <v>46099</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1507,7 +1509,7 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://es.linkedin.com/company/spektrumgrp</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -1529,7 +1531,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>li-4335125314</t>
+          <t>li-4320219168</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1539,18 +1541,18 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4335125314</t>
+          <t>https://www.linkedin.com/jobs/view/4320219168</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Consultant - Operations Excellence Program</t>
+          <t>(Senior) Consultant - Business Consulting - Finance</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1559,7 +1561,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46166</v>
+        <v>46178</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1578,7 +1580,7 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://uk.linkedin.com/company/ernstandyoung</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -1600,7 +1602,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>li-4423364166</t>
+          <t>li-4412749267</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1610,26 +1612,28 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4423364166</t>
+          <t>https://www.linkedin.com/jobs/view/4412749267</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Carhartt WIP (Work In Progress)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>46153</v>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -1647,7 +1651,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -1669,7 +1673,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>li-4416485748</t>
+          <t>li-4416601732</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1679,25 +1683,21 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416485748</t>
+          <t>https://www.linkedin.com/jobs/view/4416601732</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Drug Safety Case Manager</t>
+          <t>Manager Experis Basel</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Flexsis</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Allschwil, Basel-Country, Switzerland</t>
-        </is>
-      </c>
+          <t>Experis Switzerland</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" s="2" t="n">
         <v>46161</v>
       </c>
@@ -1718,7 +1718,7 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/flexsisch</t>
+          <t>https://ch.linkedin.com/company/experis-switzerland</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -1740,7 +1740,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>li-4417604986</t>
+          <t>li-4404786229</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1750,27 +1750,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4417604986</t>
+          <t>https://www.linkedin.com/jobs/view/4404786229</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Facility Coordinator (a) 80%</t>
+          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>JYSK</t>
+          <t>Fraunhofer IAF</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Zofingen, Aargau, Switzerland</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46170</v>
+        <v>46135</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1789,7 +1789,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/company/jysk</t>
+          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -1811,7 +1811,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4419242792</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1821,27 +1821,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4419242792</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Healthcare Consultant</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>Let's Create SUCCESS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Bern, Berne, Switzerland</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46150</v>
+        <v>46175</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1860,7 +1860,7 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://ie.linkedin.com/company/rachel-collery</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -1882,7 +1882,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>li-4320219168</t>
+          <t>li-4291106113</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1892,18 +1892,18 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4320219168</t>
+          <t>https://www.linkedin.com/jobs/view/4291106113</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>(Senior) Consultant - Business Consulting - Finance</t>
+          <t>Consultant (m/f/d) - Financial Services</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>Simon-Kucher</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46157</v>
+        <v>46178</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/ernstandyoung</t>
+          <t>https://de.linkedin.com/company/simon-kucher</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -1953,7 +1953,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>li-4335254607</t>
+          <t>li-4409306761</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1963,27 +1963,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4335254607</t>
+          <t>https://www.linkedin.com/jobs/view/4409306761</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Consultant - Procurement</t>
+          <t>Country Manager Belgium and Luxembourg (BeLux-based) 🇧🇪🇱🇺</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Chargemap</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46166</v>
+        <v>46147</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -2002,7 +2002,7 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://fr.linkedin.com/company/chargemap</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2024,7 +2024,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>li-4409306761</t>
+          <t>li-4335254607</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2034,27 +2034,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409306761</t>
+          <t>https://www.linkedin.com/jobs/view/4335254607</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Country Manager Belgium and Luxembourg (BeLux-based) 🇧🇪🇱🇺</t>
+          <t>Consultant - Procurement</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Chargemap</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46147</v>
+        <v>46166</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -2073,7 +2073,7 @@
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/chargemap</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2095,7 +2095,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>li-4414574747</t>
+          <t>li-4407827511</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2105,27 +2105,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414574747</t>
+          <t>https://www.linkedin.com/jobs/view/4407827511</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>(Junior) Strategy and Transformation Consultant</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Capgemini Invent</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Belfort, Bourgogne-Franche-Comté, France</t>
+          <t>Opfikon, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46156</v>
+        <v>46140</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -2144,7 +2144,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://fr.linkedin.com/company/capgemini-invent</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2166,7 +2166,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>li-4423364166</t>
+          <t>li-4424772167</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2176,26 +2176,28 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4423364166</t>
+          <t>https://www.linkedin.com/jobs/view/4424772167</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Sales Operations Manager</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>RealAdvisor</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>46178</v>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
@@ -2213,7 +2215,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://ch.linkedin.com/company/realadvisor-com</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2377,7 +2379,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>li-4359225027</t>
+          <t>li-4408692266</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2387,23 +2389,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359225027</t>
+          <t>https://www.linkedin.com/jobs/view/4408692266</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Strategy &amp; Operations Manager</t>
+          <t>Country Sales Manager Schweiz (mwd)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Revolut</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>CCR Commercial Refrigeration</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Pratteln, Basel-Country, Switzerland</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n">
-        <v>46166</v>
+        <v>46146</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -2422,7 +2428,7 @@
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/revolut</t>
+          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -2444,7 +2450,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>li-4408692266</t>
+          <t>li-4392923773</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2454,27 +2460,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4408692266</t>
+          <t>https://www.linkedin.com/jobs/view/4392923773</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Country Sales Manager Schweiz (mwd)</t>
+          <t>Manager/in Operations (m/w/d)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CCR Commercial Refrigeration</t>
+          <t>Thommen Group</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Pratteln, Basel-Country, Switzerland</t>
+          <t>Aarwangen, Berne, Switzerland</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46146</v>
+        <v>46111</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -2493,7 +2499,7 @@
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
+          <t>https://ch.linkedin.com/company/thommengroup</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -2515,7 +2521,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>li-4392923773</t>
+          <t>li-4400383855</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2525,27 +2531,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4392923773</t>
+          <t>https://www.linkedin.com/jobs/view/4400383855</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Manager/in Operations (m/w/d)</t>
+          <t>Senior Quality Specialist (100%)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Thommen Group</t>
+          <t>Climeworks</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Aarwangen, Berne, Switzerland</t>
+          <t>Opfikon, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46111</v>
+        <v>46165</v>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -2564,7 +2570,7 @@
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/thommengroup</t>
+          <t>https://www.linkedin.com/company/climeworks</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -2586,7 +2592,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>li-4416485748</t>
+          <t>li-4400371371</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2596,27 +2602,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416485748</t>
+          <t>https://www.linkedin.com/jobs/view/4400371371</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Drug Safety Case Manager</t>
+          <t>Senior Quality Specialist (100%)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Flexsis</t>
+          <t>Climeworks</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Allschwil, Basel-Country, Switzerland</t>
+          <t>Opfikon, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46161</v>
+        <v>46164</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -2635,7 +2641,7 @@
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/flexsisch</t>
+          <t>https://www.linkedin.com/company/climeworks</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
@@ -2728,7 +2734,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4402694276</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2738,27 +2744,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4402694276</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Family Resource Specialist</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>Children's Home &amp; Aid</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Court, Berne, Switzerland</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46150</v>
+        <v>46128</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -2777,7 +2783,7 @@
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://www.linkedin.com/company/children'shome&amp;aid</t>
         </is>
       </c>
       <c r="W32" t="inlineStr"/>
@@ -2799,7 +2805,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>li-4409247899</t>
+          <t>li-4408692266</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2809,27 +2815,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409247899</t>
+          <t>https://www.linkedin.com/jobs/view/4408692266</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Content Specialist</t>
+          <t>Country Sales Manager Schweiz (mwd)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>CCR Commercial Refrigeration</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Pratteln, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46149</v>
+        <v>46146</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -2848,7 +2854,7 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
         </is>
       </c>
       <c r="W33" t="inlineStr"/>
@@ -2870,7 +2876,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>li-4408692266</t>
+          <t>li-4407311355</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2880,27 +2886,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4408692266</t>
+          <t>https://www.linkedin.com/jobs/view/4407311355</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Country Sales Manager Schweiz (mwd)</t>
+          <t>Senior Director, Country Manager, Switzerland</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CCR Commercial Refrigeration</t>
+          <t>Revolution Medicines</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Pratteln, Basel-Country, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46146</v>
+        <v>46163</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -2919,7 +2925,7 @@
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
+          <t>https://www.linkedin.com/company/revolution-medicines</t>
         </is>
       </c>
       <c r="W34" t="inlineStr"/>
@@ -2941,7 +2947,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>li-4410009795</t>
+          <t>li-4398599784</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2951,27 +2957,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410009795</t>
+          <t>https://www.linkedin.com/jobs/view/4398599784</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Responsable Production H/F</t>
+          <t>Vice President, Business Manager</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>L’univers NOZ</t>
+          <t>AMETEK</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Reinach, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>46167</v>
+        <v>46162</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
@@ -2990,7 +2996,7 @@
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/lunivers-noz</t>
+          <t>https://www.linkedin.com/company/ametek</t>
         </is>
       </c>
       <c r="W35" t="inlineStr"/>
@@ -3012,7 +3018,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>li-4398599784</t>
+          <t>li-4420941154</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3022,27 +3028,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4398599784</t>
+          <t>https://www.linkedin.com/jobs/view/4420941154</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Vice President, Business Manager</t>
+          <t>IT Service Desk Specialist</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>AMETEK</t>
+          <t>KDR Talent Solutions</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Reinach, Basel-Country, Switzerland</t>
+          <t>Essen, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>46162</v>
+        <v>46171</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -3061,7 +3067,7 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ametek</t>
+          <t>https://uk.linkedin.com/company/kdrtalent</t>
         </is>
       </c>
       <c r="W36" t="inlineStr"/>
@@ -3083,7 +3089,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>li-4413366651</t>
+          <t>li-4416628423</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3093,27 +3099,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413366651</t>
+          <t>https://www.linkedin.com/jobs/view/4416628423</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Assistant General Manager / Assistenz der Hoteldirektion (m/w/d)</t>
+          <t>Business Consultant (m/w/d) Strategie &amp; Transformation</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Hotel Am Rathaus Freibug</t>
+          <t>Deutsche Telekom</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
-        <v>46162</v>
+        <v>46161</v>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
@@ -3132,7 +3138,7 @@
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/hotel-am-rathaus-freibug</t>
+          <t>https://de.linkedin.com/company/telekom</t>
         </is>
       </c>
       <c r="W37" t="inlineStr"/>
@@ -3154,7 +3160,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>li-4420147175</t>
+          <t>li-4412559176</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3164,18 +3170,18 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4420147175</t>
+          <t>https://www.linkedin.com/jobs/view/4412559176</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Consultant (m/w/d)</t>
+          <t>Associate - Consulting</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Bain &amp; Company</t>
+          <t>VIVALDI_</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3184,7 +3190,7 @@
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>46176</v>
+        <v>46127</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -3203,7 +3209,7 @@
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/bain-and-company</t>
+          <t>https://www.linkedin.com/company/vivaldi-group</t>
         </is>
       </c>
       <c r="W38" t="inlineStr"/>
@@ -3225,7 +3231,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>li-4301586122</t>
+          <t>li-4410012963</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3235,18 +3241,18 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4301586122</t>
+          <t>https://www.linkedin.com/jobs/view/4410012963</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Experienced Consultant - Capital Excellence</t>
+          <t>Senior Associate - Consulting</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>VIVALDI_</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3255,7 +3261,7 @@
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46176</v>
+        <v>46121</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -3274,7 +3280,7 @@
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://www.linkedin.com/company/vivaldi-group</t>
         </is>
       </c>
       <c r="W39" t="inlineStr"/>
@@ -3296,7 +3302,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>li-4301569738</t>
+          <t>li-4389002832</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3306,27 +3312,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4301569738</t>
+          <t>https://www.linkedin.com/jobs/view/4389002832</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Experienced Consultant - Capital Excellence</t>
+          <t>Management Consultant (d/f/m), DHL Consulting Europe</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>DHL</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>46173</v>
+        <v>46105</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -3345,7 +3351,7 @@
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://de.linkedin.com/company/dhl</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
@@ -3367,7 +3373,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>li-4266954854</t>
+          <t>li-4425614569</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3377,24 +3383,26 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4266954854</t>
+          <t>https://www.linkedin.com/jobs/view/4425614569</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Experienced Consultant (Düsseldorf)</t>
+          <t>Healthcare Consultant</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>OC&amp;C Strategy Consultants</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" s="2" t="n">
-        <v>46161</v>
-      </c>
+          <t>Alcimed</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
@@ -3412,7 +3420,7 @@
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/oc&amp;c-strategy-consultants</t>
+          <t>https://fr.linkedin.com/company/alcimed</t>
         </is>
       </c>
       <c r="W41" t="inlineStr"/>
@@ -3434,7 +3442,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>li-4371968232</t>
+          <t>li-4413617729</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3444,27 +3452,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4371968232</t>
+          <t>https://www.linkedin.com/jobs/view/4413617729</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Consultant (w/m/d) Public Sector</t>
+          <t>Store Manager - Cologne (m/f/d)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Horváth</t>
+          <t>LAP Coffee</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>46070</v>
+        <v>46162</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -3483,7 +3491,7 @@
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/horvathpartners</t>
+          <t>https://de.linkedin.com/company/lap-coffee</t>
         </is>
       </c>
       <c r="W42" t="inlineStr"/>
@@ -3505,7 +3513,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>li-4384316600</t>
+          <t>li-4413931472</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3515,27 +3523,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4384316600</t>
+          <t>https://www.linkedin.com/jobs/view/4413931472</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Sales Area Manager Nürnberg Würzburg (w_m_d)</t>
+          <t>Store Manager (m/w/d), Emporio Armani Düsseldorf</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Barilla Group</t>
+          <t>Giorgio Armani</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>46157</v>
+        <v>46155</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -3554,7 +3562,7 @@
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/barilla-group</t>
+          <t>https://it.linkedin.com/company/giorgio-armani</t>
         </is>
       </c>
       <c r="W43" t="inlineStr"/>
@@ -3576,7 +3584,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>li-4413931472</t>
+          <t>li-4412707731</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3586,27 +3594,23 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413931472</t>
+          <t>https://www.linkedin.com/jobs/view/4412707731</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Store Manager (m/w/d), Emporio Armani Düsseldorf</t>
+          <t>Retail Operation Manager</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Giorgio Armani</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
+          <t>Anker Innovations</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" s="2" t="n">
-        <v>46155</v>
+        <v>46153</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -3625,7 +3629,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/giorgio-armani</t>
+          <t>https://www.linkedin.com/company/ankerinnovations</t>
         </is>
       </c>
       <c r="W44" t="inlineStr"/>
@@ -3647,7 +3651,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>li-4412707731</t>
+          <t>li-4382075534</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3657,23 +3661,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412707731</t>
+          <t>https://www.linkedin.com/jobs/view/4382075534</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Retail Operation Manager</t>
+          <t>General Manager (m/w/d)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Anker Innovations</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
+          <t>Autogrill Germany</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
       <c r="H45" s="2" t="n">
-        <v>46153</v>
+        <v>46091</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -3692,7 +3700,7 @@
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ankerinnovations</t>
+          <t>https://de.linkedin.com/company/autogrill-germany</t>
         </is>
       </c>
       <c r="W45" t="inlineStr"/>
@@ -3714,7 +3722,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>li-4410039212</t>
+          <t>li-4379922140</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3724,23 +3732,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410039212</t>
+          <t>https://www.linkedin.com/jobs/view/4379922140</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Country Manager Germany</t>
+          <t>Area Manager - Cologne (m/f/d)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>DeWarmte</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
+          <t>LAP Coffee</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
       <c r="H46" s="2" t="n">
-        <v>46146</v>
+        <v>46083</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -3759,7 +3771,7 @@
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/dewarmte</t>
+          <t>https://de.linkedin.com/company/lap-coffee</t>
         </is>
       </c>
       <c r="W46" t="inlineStr"/>
@@ -3781,7 +3793,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>li-4379922140</t>
+          <t>li-4421582805</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3791,27 +3803,23 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4379922140</t>
+          <t>https://www.linkedin.com/jobs/view/4421582805</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Area Manager - Cologne (m/f/d)</t>
+          <t>Talent Advisor</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>LAP Coffee</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
+          <t>Randstad Enterprise</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" s="2" t="n">
-        <v>46083</v>
+        <v>46180</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
@@ -3830,7 +3838,7 @@
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/lap-coffee</t>
+          <t>https://nl.linkedin.com/company/randstadenterprise</t>
         </is>
       </c>
       <c r="W47" t="inlineStr"/>
@@ -3852,7 +3860,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>li-4423985038</t>
+          <t>li-4419053552</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3862,27 +3870,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4423985038</t>
+          <t>https://www.linkedin.com/jobs/view/4419053552</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BaSE Specialist (m/w/d)</t>
+          <t>Order Management Specialist</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>Octave</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H48" s="2" t="n">
-        <v>46175</v>
+        <v>46170</v>
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
@@ -3901,7 +3909,7 @@
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ups</t>
+          <t>https://www.linkedin.com/company/octaveintelligence</t>
         </is>
       </c>
       <c r="W48" t="inlineStr"/>
@@ -3923,7 +3931,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>li-4421807992</t>
+          <t>li-4413366651</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3933,27 +3941,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4421807992</t>
+          <t>https://www.linkedin.com/jobs/view/4413366651</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Revisor Specialist - Penny International (m/w/d)</t>
+          <t>Assistant General Manager / Assistenz der Hoteldirektion (m/w/d)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>PENNY International (REWE Group)</t>
+          <t>Hotel Am Rathaus Freibug</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H49" s="2" t="n">
-        <v>46174</v>
+        <v>46162</v>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
@@ -3972,7 +3980,7 @@
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/penny-international-rewe-group</t>
+          <t>https://www.linkedin.com/company/hotel-am-rathaus-freibug</t>
         </is>
       </c>
       <c r="W49" t="inlineStr"/>
@@ -3994,7 +4002,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>li-4422122505</t>
+          <t>li-4409006433</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4004,27 +4012,23 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4422122505</t>
+          <t>https://www.linkedin.com/jobs/view/4409006433</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Specialist BCM Production (m/w/d)</t>
+          <t>Employee Relations Manager (m/w/d</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Vaillant Deutschland</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Remscheid, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
+          <t>Dyson</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" s="2" t="n">
-        <v>46174</v>
+        <v>46164</v>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
@@ -4043,7 +4047,7 @@
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/vaillantdeutschland</t>
+          <t>https://sg.linkedin.com/company/dyson</t>
         </is>
       </c>
       <c r="W50" t="inlineStr"/>
@@ -4065,7 +4069,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>li-4419053552</t>
+          <t>li-4376393381</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4075,27 +4079,27 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4419053552</t>
+          <t>https://www.linkedin.com/jobs/view/4376393381</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Order Management Specialist</t>
+          <t>Assistant Manager, Procurement Consulting (m/f/d)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Octave</t>
+          <t>Interpath</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H51" s="2" t="n">
-        <v>46170</v>
+        <v>46075</v>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
@@ -4114,7 +4118,7 @@
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/octaveintelligence</t>
+          <t>https://uk.linkedin.com/company/interpathadvisory</t>
         </is>
       </c>
       <c r="W51" t="inlineStr"/>
@@ -4136,7 +4140,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>li-4416894948</t>
+          <t>li-4412848219</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4146,27 +4150,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416894948</t>
+          <t>https://www.linkedin.com/jobs/view/4412848219</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Spezialist (m/w/d) für Einlagensicherung</t>
+          <t>PostDoc: Akademische Rätin / Akademischer Rat auf Zeit (w/m/d) - Lehrstuhl für Biologische Psychologie, Klinische Psychologie und Psychotherapie</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Prüfungsverband deutscher Banken e.V.</t>
+          <t>The University of Freiburg</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H52" s="2" t="n">
-        <v>46169</v>
+        <v>46160</v>
       </c>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
@@ -4185,7 +4189,7 @@
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/pruefungsverbanddeutscherbanken</t>
+          <t>https://de.linkedin.com/school/albert-ludwigs-universitaet-freiburg/</t>
         </is>
       </c>
       <c r="W52" t="inlineStr"/>
@@ -4207,7 +4211,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>li-4419276665</t>
+          <t>li-4404077580</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4217,27 +4221,27 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4419276665</t>
+          <t>https://www.linkedin.com/jobs/view/4404077580</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Senior Analyst:in</t>
+          <t>Member of Technical Staff - Post Training</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Gi Group</t>
+          <t>Black Forest Labs</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>46175</v>
+        <v>46132</v>
       </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
@@ -4256,7 +4260,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/gi-group</t>
+          <t>https://de.linkedin.com/company/bflai</t>
         </is>
       </c>
       <c r="W53" t="inlineStr"/>
@@ -4278,7 +4282,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>li-4411718887</t>
+          <t>li-4328078441</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4288,27 +4292,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4411718887</t>
+          <t>https://www.linkedin.com/jobs/view/4328078441</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Business &amp; Customer Data Analyst</t>
+          <t>Scientist (all genders) - GaN Components, Circuits &amp; Modules</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>MCH Group</t>
+          <t>Fraunhofer Karriere</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H54" s="2" t="n">
-        <v>46150</v>
+        <v>46010</v>
       </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
@@ -4327,7 +4331,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
+          <t>https://de.linkedin.com/company/fraunhoferkarriere</t>
         </is>
       </c>
       <c r="W54" t="inlineStr"/>
@@ -4349,7 +4353,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>li-4404786229</t>
+          <t>li-4315852967</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4359,18 +4363,18 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404786229</t>
+          <t>https://www.linkedin.com/jobs/view/4315852967</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
+          <t>Member of Technical Staff - Image / Video Generation</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Fraunhofer IAF</t>
+          <t>Black Forest Labs</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4379,7 +4383,7 @@
         </is>
       </c>
       <c r="H55" s="2" t="n">
-        <v>46135</v>
+        <v>45946</v>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
@@ -4398,7 +4402,7 @@
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
+          <t>https://de.linkedin.com/company/bflai</t>
         </is>
       </c>
       <c r="W55" t="inlineStr"/>
@@ -4420,7 +4424,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>li-4414586149</t>
+          <t>li-4354401247</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4430,27 +4434,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414586149</t>
+          <t>https://www.linkedin.com/jobs/view/4354401247</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Consultant Junior Transformation des Organisations F/H</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
+          <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
       <c r="H56" s="2" t="n">
-        <v>46156</v>
+        <v>46163</v>
       </c>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
@@ -4469,7 +4473,7 @@
       <c r="U56" t="inlineStr"/>
       <c r="V56" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://www.linkedin.com/company/deloitte</t>
         </is>
       </c>
       <c r="W56" t="inlineStr"/>
@@ -4491,7 +4495,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>li-4423364166</t>
+          <t>li-4412251940</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4501,26 +4505,28 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4423364166</t>
+          <t>https://www.linkedin.com/jobs/view/4412251940</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Junior Consultant (m/w/d) Financial Consulting</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>PFP-PrivateFinancePartners GmbH</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Colmar, Grand Est, France</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr"/>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>46160</v>
+      </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
@@ -4538,7 +4544,7 @@
       <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://de.linkedin.com/company/privatefinancepartners-gmbh</t>
         </is>
       </c>
       <c r="W57" t="inlineStr"/>
@@ -4560,7 +4566,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>li-4423350822</t>
+          <t>li-4409933547</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4570,26 +4576,28 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4423350822</t>
+          <t>https://www.linkedin.com/jobs/view/4409933547</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Junior Consultant Finance – Homeoffice</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Convit Central GmbH</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
+          <t>Olten, Solothurn, Switzerland</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>46148</v>
+      </c>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
@@ -4607,7 +4615,7 @@
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://ch.linkedin.com/company/convit-central-gmbh</t>
         </is>
       </c>
       <c r="W58" t="inlineStr"/>
@@ -4629,7 +4637,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>li-4423362471</t>
+          <t>li-4386859417</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4639,18 +4647,18 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4423362471</t>
+          <t>https://www.linkedin.com/jobs/view/4386859417</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Junior Business Continuity Management Consultant</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>Spektrum</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4658,7 +4666,9 @@
           <t>Strasbourg, Grand Est, France</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" s="2" t="n">
+        <v>46099</v>
+      </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
@@ -4676,7 +4686,7 @@
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://es.linkedin.com/company/spektrumgrp</t>
         </is>
       </c>
       <c r="W59" t="inlineStr"/>
@@ -4698,7 +4708,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>li-4423343998</t>
+          <t>li-4375964465</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4708,26 +4718,28 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4423343998</t>
+          <t>https://www.linkedin.com/jobs/view/4375964465</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
+          <t>Junior Consultant 80 % – 100 % in Basel</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
+          <t>APP Unternehmensberatung AG</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr"/>
+          <t>Basel, Basel, Switzerland</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>46080</v>
+      </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
@@ -4745,7 +4757,7 @@
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/gclexperts</t>
+          <t>https://ch.linkedin.com/company/app-unternehmensberatung-ag</t>
         </is>
       </c>
       <c r="W60" t="inlineStr"/>
@@ -4767,7 +4779,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>li-4386750509</t>
+          <t>li-4385596342</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4777,27 +4789,27 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386750509</t>
+          <t>https://www.linkedin.com/jobs/view/4385596342</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Spontanbewerbung</t>
+          <t>Sales Consultant/ in 100%</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>INFORS HT</t>
+          <t>JobCourier</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Bottmingen, Basel-Country, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H61" s="2" t="n">
-        <v>46098</v>
+        <v>46095</v>
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
@@ -4816,7 +4828,7 @@
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/inforsht</t>
+          <t>https://ch.linkedin.com/company/jobcourier</t>
         </is>
       </c>
       <c r="W61" t="inlineStr"/>

</xml_diff>

<commit_message>
Update Job Report Sat Jun 13 02:34:08 UTC 2026
</commit_message>
<xml_diff>
--- a/Latest_Job_Report.xlsx
+++ b/Latest_Job_Report.xlsx
@@ -612,7 +612,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>li-4420911792</t>
+          <t>li-4413821098</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -622,27 +622,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4420911792</t>
+          <t>https://www.linkedin.com/jobs/view/4413821098</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Medical Researcher (m/w/d)</t>
+          <t>CX/UX Researcher (m/f/d) - Hybrid</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Deutsches Promotionszentrum</t>
+          <t>Wolters Kluwer</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Hürth, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46171</v>
+        <v>46176</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -661,7 +661,7 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
+          <t>https://nl.linkedin.com/company/wolters-kluwer</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -683,7 +683,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>li-4404056876</t>
+          <t>li-4408764275</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -693,27 +693,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404056876</t>
+          <t>https://www.linkedin.com/jobs/view/4408764275</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Researcher</t>
+          <t>Quantitative Researcher / Statistiker/ Data Analyst (m/w/d)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The IN Group</t>
+          <t>Deutsches Promotionszentrum</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Basel, Switzerland</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46170</v>
+        <v>46142</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -732,7 +732,7 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/we-are-tig</t>
+          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -754,7 +754,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>li-4413525792</t>
+          <t>li-4414022207</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -764,24 +764,26 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413525792</t>
+          <t>https://www.linkedin.com/jobs/view/4414022207</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Market Researcher</t>
+          <t>Applied Researcher</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Xiaomi Technology</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" s="2" t="n">
-        <v>46154</v>
-      </c>
+          <t>eBay</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Aachen, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -799,7 +801,7 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://cn.linkedin.com/company/xiaomi-technology</t>
+          <t>https://www.linkedin.com/company/ebay</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -821,7 +823,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>li-4407397044</t>
+          <t>li-4414008551</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -831,28 +833,26 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407397044</t>
+          <t>https://www.linkedin.com/jobs/view/4414008551</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Medical researcher (MD., m/f/div) (m/w/div.)</t>
+          <t>Senior Applied Researcher</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Deutsches Diabetes-Zentrum</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>46142</v>
-      </c>
+          <t>Aachen, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -870,7 +870,7 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-diabetes-zentrum</t>
+          <t>https://www.linkedin.com/company/ebay</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -892,7 +892,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>li-4257970631</t>
+          <t>li-4414173590</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -902,27 +902,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4257970631</t>
+          <t>https://www.linkedin.com/jobs/view/4414173590</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Research Assistant/Doctoral Student (f/m/d) - Chair of Production Management</t>
+          <t>Investment Research Analyst | Upto $100/hr</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>WHU Entrepreneurship Roundtable</t>
+          <t>Mercor</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Vallendar, Rhineland-Palatinate, Germany</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>45813</v>
+        <v>46155</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -941,7 +941,7 @@
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/whu-entrepreneurship-roundtable</t>
+          <t>https://www.linkedin.com/company/mercor-ai</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -963,7 +963,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>li-4418110532</t>
+          <t>li-4404056876</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -973,27 +973,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4418110532</t>
+          <t>https://www.linkedin.com/jobs/view/4404056876</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Medical Researcher (m/w/d)</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Deutsches Promotionszentrum</t>
+          <t>The IN Group</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46164</v>
+        <v>46170</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deutsches-promotionszentrum</t>
+          <t>https://uk.linkedin.com/company/we-are-tig</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>li-4414173590</t>
+          <t>li-4404056876</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1044,27 +1044,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4414173590</t>
+          <t>https://www.linkedin.com/jobs/view/4404056876</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Investment Research Analyst | Upto $100/hr</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>The IN Group</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46155</v>
+        <v>46170</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1083,7 +1083,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://uk.linkedin.com/company/we-are-tig</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1105,7 +1105,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4407427079</t>
+          <t>li-4422260598</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1115,27 +1115,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407427079</t>
+          <t>https://www.linkedin.com/jobs/view/4422260598</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Research Scientist, Foundation Model</t>
+          <t>Senior Business/Data Modelling Analyst</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Prior Labs</t>
+          <t>Glocomms</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46139</v>
+        <v>46182</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -1154,7 +1154,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/prior-labs</t>
+          <t>https://www.linkedin.com/company/glocomms</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1170,13 +1170,13 @@
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4415995749</t>
+          <t>li-4422260598</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1186,27 +1186,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4415995749</t>
+          <t>https://www.linkedin.com/jobs/view/4422260598</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Investment Research Analyst</t>
+          <t>Senior Business/Data Modelling Analyst</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>Glocomms</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46162</v>
+        <v>46182</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1225,7 +1225,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mercor-ai</t>
+          <t>https://www.linkedin.com/company/glocomms</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1241,13 +1241,13 @@
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4417613007</t>
+          <t>li-4422265990</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1257,27 +1257,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4417613007</t>
+          <t>https://www.linkedin.com/jobs/view/4422265990</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Research Associate - Chemistry</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>UNSW</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46170</v>
+        <v>46182</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1296,7 +1296,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://au.linkedin.com/school/unsw/</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1312,13 +1312,13 @@
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4386853728</t>
+          <t>li-4423125971</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1328,27 +1328,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386853728</t>
+          <t>https://www.linkedin.com/jobs/view/4423125971</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Network Specialist</t>
+          <t>Facility Coordinator (a) 80%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Spektrum</t>
+          <t>JYSK</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Zofingen, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46100</v>
+        <v>46183</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1367,7 +1367,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://es.linkedin.com/company/spektrumgrp</t>
+          <t>https://dk.linkedin.com/company/jysk</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1389,7 +1389,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>li-4380147309</t>
+          <t>li-4422265990</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1399,27 +1399,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4380147309</t>
+          <t>https://www.linkedin.com/jobs/view/4422265990</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>KONSTANZ - Kundenservice / Station Service Specialist (m/w/d)</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>roadsurfer</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Aach, Baden-Württemberg, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46084</v>
+        <v>46182</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1438,7 +1438,7 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/roadsurfer-gmbh</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -1460,7 +1460,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>li-4386868249</t>
+          <t>li-4427570317</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1470,27 +1470,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386868249</t>
+          <t>https://www.linkedin.com/jobs/view/4427570317</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Continuous Service Improvement Specialist</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Spektrum</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Colmar, Grand Est, France</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46099</v>
+        <v>46184</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1509,7 +1509,7 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://es.linkedin.com/company/spektrumgrp</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -1531,7 +1531,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>li-4320219168</t>
+          <t>li-4427570317</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1541,27 +1541,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4320219168</t>
+          <t>https://www.linkedin.com/jobs/view/4427570317</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(Senior) Consultant - Business Consulting - Finance</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Colmar, Grand Est, France</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46178</v>
+        <v>46184</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1580,7 +1580,7 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/ernstandyoung</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -1602,7 +1602,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>li-4412749267</t>
+          <t>li-4427186272</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1612,27 +1612,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412749267</t>
+          <t>https://www.linkedin.com/jobs/view/4427186272</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Customer Service E-Commerce Coordinator (m/w/d)</t>
+          <t>Communication and Change Coordinator</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Carhartt WIP (Work In Progress)</t>
+          <t>Proclinical Staffing</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Weil am Rhein, Baden-Württemberg, Germany</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46153</v>
+        <v>46184</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1651,7 +1651,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/carhartt-work-in-progress</t>
+          <t>https://uk.linkedin.com/company/proclinical-staffing</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -1673,7 +1673,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>li-4416601732</t>
+          <t>li-4409306761</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1683,23 +1683,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416601732</t>
+          <t>https://www.linkedin.com/jobs/view/4409306761</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Manager Experis Basel</t>
+          <t>Country Manager Belgium and Luxembourg (BeLux-based) 🇧🇪🇱🇺</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Experis Switzerland</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>Chargemap</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Strasbourg, Grand Est, France</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="n">
-        <v>46161</v>
+        <v>46147</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1718,7 +1722,7 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/experis-switzerland</t>
+          <t>https://fr.linkedin.com/company/chargemap</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -1811,7 +1815,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>li-4419242792</t>
+          <t>li-4320219168</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1821,27 +1825,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4419242792</t>
+          <t>https://www.linkedin.com/jobs/view/4320219168</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Healthcare Consultant</t>
+          <t>(Senior) Consultant - Business Consulting - Finance</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Let's Create SUCCESS</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Bern, Berne, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1860,7 +1864,7 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://ie.linkedin.com/company/rachel-collery</t>
+          <t>https://uk.linkedin.com/company/ernstandyoung</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -1882,7 +1886,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>li-4291106113</t>
+          <t>li-4427575287</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1892,27 +1896,27 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4291106113</t>
+          <t>https://www.linkedin.com/jobs/view/4427575287</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Consultant (m/f/d) - Financial Services</t>
+          <t>CONSULTANT EN GESTION D'ENTREPRISE</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Simon-Kucher</t>
+          <t>GCL - l'innovation dans l'accompagnement des entreprises</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Colmar, Grand Est, France</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46178</v>
+        <v>46184</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1931,7 +1935,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/simon-kucher</t>
+          <t>https://fr.linkedin.com/company/gclexperts</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -1953,7 +1957,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>li-4409306761</t>
+          <t>li-4421963128</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1963,27 +1967,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409306761</t>
+          <t>https://www.linkedin.com/jobs/view/4421963128</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Country Manager Belgium and Luxembourg (BeLux-based) 🇧🇪🇱🇺</t>
+          <t>SENIOR COMMERCIAL MANAGER USA (FMCG)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Chargemap</t>
+          <t>MaserGrup</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46147</v>
+        <v>46181</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -2002,7 +2006,7 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/chargemap</t>
+          <t>https://es.linkedin.com/company/serveis-i-administracions-masergrup-sl</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2166,7 +2170,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>li-4424772167</t>
+          <t>li-4398599784</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2176,27 +2180,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4424772167</t>
+          <t>https://www.linkedin.com/jobs/view/4398599784</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sales Operations Manager</t>
+          <t>Vice President, Business Manager</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RealAdvisor</t>
+          <t>AMETEK</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Reinach, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46178</v>
+        <v>46184</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -2215,7 +2219,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/realadvisor-com</t>
+          <t>https://www.linkedin.com/company/ametek</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2237,7 +2241,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>li-4422364081</t>
+          <t>li-4424772167</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2247,27 +2251,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4422364081</t>
+          <t>https://www.linkedin.com/jobs/view/4424772167</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Responsable de magasin  H/F</t>
+          <t>Sales Operations Manager</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>BLACKSTORE France</t>
+          <t>RealAdvisor</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Saint-Louis, Grand Est, France</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -2286,7 +2290,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/blackstore</t>
+          <t>https://ch.linkedin.com/company/realadvisor-com</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -2308,7 +2312,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>li-4416856371</t>
+          <t>li-4422364081</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2318,27 +2322,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416856371</t>
+          <t>https://www.linkedin.com/jobs/view/4422364081</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Filialleiter:in / Store Manager 100% - Basel</t>
+          <t>Responsable de magasin  H/F</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Veloplus AG</t>
+          <t>BLACKSTORE France</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Saint-Louis, Grand Est, France</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46168</v>
+        <v>46175</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -2357,7 +2361,7 @@
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/veloplus-ag</t>
+          <t>https://fr.linkedin.com/company/blackstore</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -2379,7 +2383,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>li-4408692266</t>
+          <t>li-4416856371</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2389,27 +2393,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4408692266</t>
+          <t>https://www.linkedin.com/jobs/view/4416856371</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Country Sales Manager Schweiz (mwd)</t>
+          <t>Filialleiter:in / Store Manager 100% - Basel</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CCR Commercial Refrigeration</t>
+          <t>Veloplus AG</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Pratteln, Basel-Country, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46146</v>
+        <v>46168</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -2428,7 +2432,7 @@
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
+          <t>https://ch.linkedin.com/company/veloplus-ag</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -2450,7 +2454,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>li-4392923773</t>
+          <t>li-4408692266</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2460,27 +2464,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4392923773</t>
+          <t>https://www.linkedin.com/jobs/view/4408692266</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Manager/in Operations (m/w/d)</t>
+          <t>Country Sales Manager Schweiz (mwd)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Thommen Group</t>
+          <t>CCR Commercial Refrigeration</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Aarwangen, Berne, Switzerland</t>
+          <t>Pratteln, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46111</v>
+        <v>46146</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -2499,7 +2503,7 @@
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/thommengroup</t>
+          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -2521,7 +2525,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>li-4400383855</t>
+          <t>li-4427186272</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2531,27 +2535,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4400383855</t>
+          <t>https://www.linkedin.com/jobs/view/4427186272</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Quality Specialist (100%)</t>
+          <t>Communication and Change Coordinator</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Climeworks</t>
+          <t>Proclinical Staffing</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Opfikon, Zurich, Switzerland</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46165</v>
+        <v>46184</v>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -2570,7 +2574,7 @@
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/climeworks</t>
+          <t>https://uk.linkedin.com/company/proclinical-staffing</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -2592,7 +2596,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>li-4400371371</t>
+          <t>li-4427016732</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2602,27 +2606,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4400371371</t>
+          <t>https://www.linkedin.com/jobs/view/4427016732</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Quality Specialist (100%)</t>
+          <t>Communications &amp; Change Coordinator</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Climeworks</t>
+          <t>Panda International</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Opfikon, Zurich, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46164</v>
+        <v>46183</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -2641,7 +2645,7 @@
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/climeworks</t>
+          <t>https://nl.linkedin.com/company/panda-international</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
@@ -2663,7 +2667,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>li-4412749267</t>
+          <t>li-4423128106</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2673,7 +2677,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412749267</t>
+          <t>https://www.linkedin.com/jobs/view/4423128106</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -2693,7 +2697,7 @@
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46153</v>
+        <v>46183</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -2734,7 +2738,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>li-4402694276</t>
+          <t>li-4427024525</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2744,27 +2748,23 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4402694276</t>
+          <t>https://www.linkedin.com/jobs/view/4427024525</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Family Resource Specialist</t>
+          <t>Communications &amp; Change Coordinator</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Children's Home &amp; Aid</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Court, Berne, Switzerland</t>
-        </is>
-      </c>
+          <t>Aston Carter</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" s="2" t="n">
-        <v>46128</v>
+        <v>46183</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -2783,7 +2783,7 @@
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/children'shome&amp;aid</t>
+          <t>https://www.linkedin.com/company/aston-carter</t>
         </is>
       </c>
       <c r="W32" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>li-4408692266</t>
+          <t>li-4413366651</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2815,27 +2815,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4408692266</t>
+          <t>https://www.linkedin.com/jobs/view/4413366651</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Country Sales Manager Schweiz (mwd)</t>
+          <t>Assistant General Manager / Assistenz der Hoteldirektion (m/w/d)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CCR Commercial Refrigeration</t>
+          <t>Hotel Am Rathaus Freibug</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Pratteln, Basel-Country, Switzerland</t>
+          <t>Freiburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46146</v>
+        <v>46162</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -2854,7 +2854,7 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ccr-commercial-refrigeration</t>
+          <t>https://www.linkedin.com/company/hotel-am-rathaus-freibug</t>
         </is>
       </c>
       <c r="W33" t="inlineStr"/>
@@ -2876,7 +2876,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>li-4407311355</t>
+          <t>li-4398599784</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2886,27 +2886,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4407311355</t>
+          <t>https://www.linkedin.com/jobs/view/4398599784</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior Director, Country Manager, Switzerland</t>
+          <t>Vice President, Business Manager</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Revolution Medicines</t>
+          <t>AMETEK</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Reinach, Basel-Country, Switzerland</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46163</v>
+        <v>46184</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -2925,7 +2925,7 @@
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/revolution-medicines</t>
+          <t>https://www.linkedin.com/company/ametek</t>
         </is>
       </c>
       <c r="W34" t="inlineStr"/>
@@ -2947,7 +2947,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>li-4398599784</t>
+          <t>li-4425999727</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2957,27 +2957,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4398599784</t>
+          <t>https://www.linkedin.com/jobs/view/4425999727</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Vice President, Business Manager</t>
+          <t>Department Manager (m/w/d) - Shoppi Tivoli / Spreitenbach (100% / 38.5 Wochenstunden)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AMETEK</t>
+          <t>H&amp;M</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Reinach, Basel-Country, Switzerland</t>
+          <t>Spreitenbach, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>46162</v>
+        <v>46182</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
@@ -2996,7 +2996,7 @@
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ametek</t>
+          <t>https://se.linkedin.com/company/h&amp;m</t>
         </is>
       </c>
       <c r="W35" t="inlineStr"/>
@@ -3018,7 +3018,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>li-4420941154</t>
+          <t>li-4422273233</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3028,27 +3028,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4420941154</t>
+          <t>https://www.linkedin.com/jobs/view/4422273233</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>IT Service Desk Specialist</t>
+          <t>Sap Finance Control Consultant</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>KDR Talent Solutions</t>
+          <t>DSR Global</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Essen, North Rhine-Westphalia, Germany</t>
+          <t>Bonn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>46171</v>
+        <v>46182</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -3067,7 +3067,7 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/kdrtalent</t>
+          <t>https://uk.linkedin.com/company/dsr-global</t>
         </is>
       </c>
       <c r="W36" t="inlineStr"/>
@@ -3089,7 +3089,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>li-4416628423</t>
+          <t>li-4266954854</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3099,27 +3099,23 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4416628423</t>
+          <t>https://www.linkedin.com/jobs/view/4266954854</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Business Consultant (m/w/d) Strategie &amp; Transformation</t>
+          <t>Experienced Consultant (Düsseldorf)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Deutsche Telekom</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
+          <t>OC&amp;C Strategy Consultants</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" s="2" t="n">
-        <v>46161</v>
+        <v>46183</v>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
@@ -3138,7 +3134,7 @@
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/telekom</t>
+          <t>https://uk.linkedin.com/company/oc&amp;c-strategy-consultants</t>
         </is>
       </c>
       <c r="W37" t="inlineStr"/>
@@ -3160,7 +3156,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>li-4412559176</t>
+          <t>li-4420147175</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3170,18 +3166,18 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412559176</t>
+          <t>https://www.linkedin.com/jobs/view/4420147175</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Associate - Consulting</t>
+          <t>Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VIVALDI_</t>
+          <t>Bain &amp; Company</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3190,7 +3186,7 @@
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>46127</v>
+        <v>46176</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -3209,7 +3205,7 @@
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/vivaldi-group</t>
+          <t>https://www.linkedin.com/company/bain-and-company</t>
         </is>
       </c>
       <c r="W38" t="inlineStr"/>
@@ -3231,7 +3227,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>li-4410012963</t>
+          <t>li-4301586122</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3241,18 +3237,18 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4410012963</t>
+          <t>https://www.linkedin.com/jobs/view/4301586122</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Senior Associate - Consulting</t>
+          <t>Experienced Consultant - Capital Excellence</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VIVALDI_</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3261,7 +3257,7 @@
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46121</v>
+        <v>46176</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -3280,7 +3276,7 @@
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/vivaldi-group</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W39" t="inlineStr"/>
@@ -3302,7 +3298,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>li-4389002832</t>
+          <t>li-4301569738</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3312,27 +3308,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4389002832</t>
+          <t>https://www.linkedin.com/jobs/view/4301569738</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Management Consultant (d/f/m), DHL Consulting Europe</t>
+          <t>Experienced Consultant - Capital Excellence</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>DHL</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>46105</v>
+        <v>46173</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -3351,7 +3347,7 @@
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/dhl</t>
+          <t>https://www.linkedin.com/company/mckinsey</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
@@ -3373,7 +3369,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>li-4425614569</t>
+          <t>li-4371968232</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3383,26 +3379,28 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4425614569</t>
+          <t>https://www.linkedin.com/jobs/view/4371968232</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Healthcare Consultant</t>
+          <t>Consultant (w/m/d) Public Sector</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Alcimed</t>
+          <t>Horváth</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
+          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
@@ -3420,7 +3418,7 @@
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/alcimed</t>
+          <t>https://de.linkedin.com/company/horvathpartners</t>
         </is>
       </c>
       <c r="W41" t="inlineStr"/>
@@ -3442,7 +3440,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>li-4413617729</t>
+          <t>li-4425602682</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3452,27 +3450,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413617729</t>
+          <t>https://www.linkedin.com/jobs/view/4425602682</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Store Manager - Cologne (m/f/d)</t>
+          <t>Global Marketing Manager (m/f/d)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>LAP Coffee</t>
+          <t>J.M. Huber Corporation</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Cologne, North Rhine-Westphalia, Germany</t>
+          <t>Bergheim, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>46162</v>
+        <v>46181</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -3491,7 +3489,7 @@
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/lap-coffee</t>
+          <t>https://www.linkedin.com/company/j.m.-huber-corporation</t>
         </is>
       </c>
       <c r="W42" t="inlineStr"/>
@@ -3513,7 +3511,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>li-4413931472</t>
+          <t>li-4413617729</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3523,27 +3521,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413931472</t>
+          <t>https://www.linkedin.com/jobs/view/4413617729</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Store Manager (m/w/d), Emporio Armani Düsseldorf</t>
+          <t>Store Manager - Cologne (m/f/d)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Giorgio Armani</t>
+          <t>LAP Coffee</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Düsseldorf, North Rhine-Westphalia, Germany</t>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>46155</v>
+        <v>46162</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -3562,7 +3560,7 @@
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>https://it.linkedin.com/company/giorgio-armani</t>
+          <t>https://de.linkedin.com/company/lap-coffee</t>
         </is>
       </c>
       <c r="W43" t="inlineStr"/>
@@ -3584,7 +3582,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>li-4412707731</t>
+          <t>li-4382075534</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3594,23 +3592,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412707731</t>
+          <t>https://www.linkedin.com/jobs/view/4382075534</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Retail Operation Manager</t>
+          <t>General Manager (m/w/d)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Anker Innovations</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
+          <t>Autogrill Germany</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Cologne, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
       <c r="H44" s="2" t="n">
-        <v>46153</v>
+        <v>46091</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -3629,7 +3631,7 @@
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ankerinnovations</t>
+          <t>https://de.linkedin.com/company/autogrill-germany</t>
         </is>
       </c>
       <c r="W44" t="inlineStr"/>
@@ -3651,7 +3653,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>li-4382075534</t>
+          <t>li-4379922140</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3661,18 +3663,18 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4382075534</t>
+          <t>https://www.linkedin.com/jobs/view/4379922140</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>General Manager (m/w/d)</t>
+          <t>Area Manager - Cologne (m/f/d)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Autogrill Germany</t>
+          <t>LAP Coffee</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3681,7 +3683,7 @@
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>46091</v>
+        <v>46083</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -3700,7 +3702,7 @@
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/autogrill-germany</t>
+          <t>https://de.linkedin.com/company/lap-coffee</t>
         </is>
       </c>
       <c r="W45" t="inlineStr"/>
@@ -3722,7 +3724,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>li-4379922140</t>
+          <t>li-3889417111</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3732,18 +3734,18 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4379922140</t>
+          <t>https://www.linkedin.com/jobs/view/3889417111</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Area Manager - Cologne (m/f/d)</t>
+          <t>STORE MANAGER</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>LAP Coffee</t>
+          <t>Copenhagen Coffee Lab</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3752,7 +3754,7 @@
         </is>
       </c>
       <c r="H46" s="2" t="n">
-        <v>46083</v>
+        <v>45391</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -3771,7 +3773,7 @@
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/lap-coffee</t>
+          <t>https://dk.linkedin.com/company/cphcoffeelab</t>
         </is>
       </c>
       <c r="W46" t="inlineStr"/>
@@ -3793,7 +3795,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>li-4421582805</t>
+          <t>li-4426343309</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3803,23 +3805,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4421582805</t>
+          <t>https://www.linkedin.com/jobs/view/4426343309</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Talent Advisor</t>
+          <t>ERP Functional Consultant (m/f/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Randstad Enterprise</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
+          <t>Redcare Pharmacy</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Mönchengladbach, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
       <c r="H47" s="2" t="n">
-        <v>46180</v>
+        <v>46182</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
@@ -3838,7 +3844,7 @@
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/randstadenterprise</t>
+          <t>https://nl.linkedin.com/company/redcare-pharmacy-com</t>
         </is>
       </c>
       <c r="W47" t="inlineStr"/>
@@ -3860,7 +3866,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>li-4419053552</t>
+          <t>li-4426305685</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3870,27 +3876,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4419053552</t>
+          <t>https://www.linkedin.com/jobs/view/4426305685</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Order Management Specialist</t>
+          <t>Senior Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Octave</t>
+          <t>ENLITE Management &amp; Engineering GmbH</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Bonn, North Rhine-Westphalia, Germany</t>
+          <t>Essen, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H48" s="2" t="n">
-        <v>46170</v>
+        <v>46182</v>
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
@@ -3909,7 +3915,7 @@
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/octaveintelligence</t>
+          <t>https://de.linkedin.com/company/enlite-gmbh</t>
         </is>
       </c>
       <c r="W48" t="inlineStr"/>
@@ -3931,7 +3937,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>li-4413366651</t>
+          <t>li-4418136274</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3941,27 +3947,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4413366651</t>
+          <t>https://www.linkedin.com/jobs/view/4418136274</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Assistant General Manager / Assistenz der Hoteldirektion (m/w/d)</t>
+          <t>Scientist in-vitro Pharmacology (m/f/d)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Hotel Am Rathaus Freibug</t>
+          <t>Grünenthal Group</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Aachen, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="H49" s="2" t="n">
-        <v>46162</v>
+        <v>46171</v>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
@@ -3980,7 +3986,7 @@
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/hotel-am-rathaus-freibug</t>
+          <t>https://de.linkedin.com/company/gruenenthal</t>
         </is>
       </c>
       <c r="W49" t="inlineStr"/>
@@ -4002,7 +4008,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>li-4409006433</t>
+          <t>li-4426303928</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4012,23 +4018,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409006433</t>
+          <t>https://www.linkedin.com/jobs/view/4426303928</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Employee Relations Manager (m/w/d</t>
+          <t>SAP Business Analyst</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Dyson</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr"/>
+          <t>Pertemps ERP (part of Network EMEA)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Aachen, North Rhine-Westphalia, Germany</t>
+        </is>
+      </c>
       <c r="H50" s="2" t="n">
-        <v>46164</v>
+        <v>46182</v>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
@@ -4047,7 +4057,7 @@
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr">
         <is>
-          <t>https://sg.linkedin.com/company/dyson</t>
+          <t>https://uk.linkedin.com/company/pertemps-erp</t>
         </is>
       </c>
       <c r="W50" t="inlineStr"/>
@@ -4140,7 +4150,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>li-4412848219</t>
+          <t>li-4422265990</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4150,27 +4160,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412848219</t>
+          <t>https://www.linkedin.com/jobs/view/4422265990</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>PostDoc: Akademische Rätin / Akademischer Rat auf Zeit (w/m/d) - Lehrstuhl für Biologische Psychologie, Klinische Psychologie und Psychotherapie</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>The University of Freiburg</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H52" s="2" t="n">
-        <v>46160</v>
+        <v>46182</v>
       </c>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
@@ -4189,7 +4199,7 @@
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/school/albert-ludwigs-universitaet-freiburg/</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W52" t="inlineStr"/>
@@ -4211,7 +4221,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>li-4404077580</t>
+          <t>li-4422260598</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4221,27 +4231,27 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4404077580</t>
+          <t>https://www.linkedin.com/jobs/view/4422260598</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - Post Training</t>
+          <t>Senior Business/Data Modelling Analyst</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Black Forest Labs</t>
+          <t>Glocomms</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Basel, Basel, Switzerland</t>
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>46132</v>
+        <v>46182</v>
       </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
@@ -4260,7 +4270,7 @@
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/bflai</t>
+          <t>https://www.linkedin.com/company/glocomms</t>
         </is>
       </c>
       <c r="W53" t="inlineStr"/>
@@ -4282,7 +4292,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>li-4328078441</t>
+          <t>li-4419276665</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4292,27 +4302,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4328078441</t>
+          <t>https://www.linkedin.com/jobs/view/4419276665</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Scientist (all genders) - GaN Components, Circuits &amp; Modules</t>
+          <t>Senior Analyst:in</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Fraunhofer Karriere</t>
+          <t>Gi Group</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H54" s="2" t="n">
-        <v>46010</v>
+        <v>46175</v>
       </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
@@ -4331,7 +4341,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/fraunhoferkarriere</t>
+          <t>https://it.linkedin.com/company/gi-group</t>
         </is>
       </c>
       <c r="W54" t="inlineStr"/>
@@ -4353,7 +4363,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>li-4315852967</t>
+          <t>li-4404786229</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4363,18 +4373,18 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4315852967</t>
+          <t>https://www.linkedin.com/jobs/view/4404786229</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - Image / Video Generation</t>
+          <t>Wissenschaftler (all genders) für MOCVD-Epitaxie mit Schwerpunkt Galliumnitrid</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Black Forest Labs</t>
+          <t>Fraunhofer IAF</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4383,7 +4393,7 @@
         </is>
       </c>
       <c r="H55" s="2" t="n">
-        <v>45946</v>
+        <v>46135</v>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
@@ -4402,7 +4412,7 @@
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/bflai</t>
+          <t>https://de.linkedin.com/company/fraunhofer-iaf</t>
         </is>
       </c>
       <c r="W55" t="inlineStr"/>
@@ -4424,7 +4434,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>li-4354401247</t>
+          <t>li-4423654256</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4434,27 +4444,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4354401247</t>
+          <t>https://www.linkedin.com/jobs/view/4423654256</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Consultant Junior Transformation des Organisations F/H</t>
+          <t>Business Consultant (m/w/d)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Markant Gruppe</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Offenburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H56" s="2" t="n">
-        <v>46163</v>
+        <v>46184</v>
       </c>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
@@ -4473,7 +4483,7 @@
       <c r="U56" t="inlineStr"/>
       <c r="V56" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deloitte</t>
+          <t>https://ch.linkedin.com/company/markant-group</t>
         </is>
       </c>
       <c r="W56" t="inlineStr"/>
@@ -4495,7 +4505,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>li-4412251940</t>
+          <t>li-4417223686</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4505,27 +4515,27 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4412251940</t>
+          <t>https://www.linkedin.com/jobs/view/4417223686</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Junior Consultant (m/w/d) Financial Consulting</t>
+          <t>AI Consultant (100%) (m/w/d), Deutschland</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>PFP-PrivateFinancePartners GmbH</t>
+          <t>HICO Group AG</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Freiburg, Baden-Württemberg, Germany</t>
+          <t>Singen, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46160</v>
+        <v>46169</v>
       </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
@@ -4544,7 +4554,7 @@
       <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/privatefinancepartners-gmbh</t>
+          <t>https://ch.linkedin.com/company/highcoordination-gmbh</t>
         </is>
       </c>
       <c r="W57" t="inlineStr"/>
@@ -4566,7 +4576,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>li-4409933547</t>
+          <t>li-4411712224</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4576,27 +4586,27 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4409933547</t>
+          <t>https://www.linkedin.com/jobs/view/4411712224</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Junior Consultant Finance – Homeoffice</t>
+          <t>AI Solution Consultant (w/m/d)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Convit Central GmbH</t>
+          <t>Bechtle</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Olten, Solothurn, Switzerland</t>
+          <t>Villingen-Schwenningen, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H58" s="2" t="n">
-        <v>46148</v>
+        <v>46150</v>
       </c>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
@@ -4615,7 +4625,7 @@
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/convit-central-gmbh</t>
+          <t>https://de.linkedin.com/company/bechtle</t>
         </is>
       </c>
       <c r="W58" t="inlineStr"/>
@@ -4637,7 +4647,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>li-4386859417</t>
+          <t>li-4410079290</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4647,27 +4657,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386859417</t>
+          <t>https://www.linkedin.com/jobs/view/4410079290</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Junior Business Continuity Management Consultant</t>
+          <t>Consultant (m/w/d) Compensation &amp; Benefits</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Spektrum</t>
+          <t>Hansgrohe Group</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Strasbourg, Grand Est, France</t>
+          <t>Offenburg, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H59" s="2" t="n">
-        <v>46099</v>
+        <v>46146</v>
       </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
@@ -4686,7 +4696,7 @@
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr">
         <is>
-          <t>https://es.linkedin.com/company/spektrumgrp</t>
+          <t>https://de.linkedin.com/company/hansgrohe-group</t>
         </is>
       </c>
       <c r="W59" t="inlineStr"/>
@@ -4708,7 +4718,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>li-4375964465</t>
+          <t>li-4289303675</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4718,27 +4728,27 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4375964465</t>
+          <t>https://www.linkedin.com/jobs/view/4289303675</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Junior Consultant 80 % – 100 % in Basel</t>
+          <t>PLM Consultant (w|m|d)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>APP Unternehmensberatung AG</t>
+          <t>BCT Technology GmbH</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Willstätt, Baden-Württemberg, Germany</t>
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>46080</v>
+        <v>45890</v>
       </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
@@ -4757,7 +4767,7 @@
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/app-unternehmensberatung-ag</t>
+          <t>https://ch.linkedin.com/company/bct-technology-gmbh</t>
         </is>
       </c>
       <c r="W60" t="inlineStr"/>
@@ -4779,7 +4789,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>li-4385596342</t>
+          <t>li-4422265990</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4789,27 +4799,27 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4385596342</t>
+          <t>https://www.linkedin.com/jobs/view/4422265990</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Sales Consultant/ in 100%</t>
+          <t>Business &amp; Customer Data Analyst</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>JobCourier</t>
+          <t>MCH Group</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Basel, Basel, Switzerland</t>
+          <t>Basel, Switzerland</t>
         </is>
       </c>
       <c r="H61" s="2" t="n">
-        <v>46095</v>
+        <v>46182</v>
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
@@ -4828,7 +4838,7 @@
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/jobcourier</t>
+          <t>https://ch.linkedin.com/company/mch-group-ltd-</t>
         </is>
       </c>
       <c r="W61" t="inlineStr"/>

</xml_diff>